<commit_message>
made ui to work on browser
</commit_message>
<xml_diff>
--- a/task_reports.xlsx
+++ b/task_reports.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\semyon-work\task-report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\semyONEX\semyon-not-work-lol\AI_ML_programmming\self_created_projects\task-report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E18DB5D-DFC4-42BC-8451-67343C816602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B60CF487-056E-406D-B738-61A3DBC700AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="370">
   <si>
     <t>Date-Time</t>
   </si>
@@ -914,7 +914,13 @@
     <t>Built a Google Sheets weekly timesheet with 5-minute time dropdowns (07:00 onward) for Start/End times that automatically calculate and sum each person's worked hours in the SUMMARY column.</t>
   </si>
   <si>
+    <t>23/06/2026 14:27:00</t>
+  </si>
+  <si>
     <t>fixed the google sheets dropdown button time setting issue, made it robust and flexible</t>
+  </si>
+  <si>
+    <t>24/06/2026 14:27:00</t>
   </si>
   <si>
     <t>created and deployed amazon s3 bucket import automation for images to have urls on the other pc, just need to set amazon cridentials using terminal and one pc left to do the same task</t>
@@ -1008,6 +1014,9 @@
 finished article translator workflow's ai agents prompts, code nodes, output parsers, all workflow is now tested, validated and deployed, now its translating in 7 different languages correctly and sends the webhook respons back correctly.</t>
   </si>
   <si>
+    <t>10/07/2026 15:01:22</t>
+  </si>
+  <si>
     <t>madedid meeting with the ctw, clarificated and managed tasks presenting and continued tasks for te day</t>
   </si>
   <si>
@@ -1033,10 +1042,16 @@
 2. new animation when level up and badges getting</t>
   </si>
   <si>
+    <t>16/07/2026 14:52:21</t>
+  </si>
+  <si>
     <t>Tested, validated and deployed the new badges and level animation feature.
 Added new ui updates on the onex-academy website project.</t>
   </si>
   <si>
+    <t>17/07/2026 14:52:21</t>
+  </si>
+  <si>
     <t>started owrking on onex-academy project website's mobile version</t>
   </si>
   <si>
@@ -1095,6 +1110,9 @@
   <si>
     <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project.
 Found some models to test with, created nice ui for browsing mp3 onex calls and model, and testing it locally.</t>
+  </si>
+  <si>
+    <t>30/07/2026 14:32:43</t>
   </si>
   <si>
     <t>In onex-academy replaced Telegram deep-link signup with a hashed six-digit confirmation code. Added confirm-password field showing a live check or cross icon. Code shipped to main; remaining blocker is the unapplied live migration.</t>
@@ -1148,9 +1166,15 @@
 Pipeline runs end-to-end; first blog failed QA on hallucinated SEO.</t>
   </si>
   <si>
+    <t>11/08/2026 15:59:35</t>
+  </si>
+  <si>
     <t>Confirmed Tilda has no write API; built three export routes instead.
 Shipped image offloading, publishing, SSR pages, hub block, HTML export.
 Rewrote nodes 10, 13, 17 around your proven Avengers page format.</t>
+  </si>
+  <si>
+    <t>12/08/2026 16:00:00</t>
   </si>
   <si>
     <t>updated the onex ai blog autiamtmaker's automation and showed to the corresponding professional</t>
@@ -1201,6 +1225,9 @@
 Password fields got show/hide eye and copy buttons</t>
   </si>
   <si>
+    <t>19/08/2026 15:21:00</t>
+  </si>
+  <si>
     <t>1. Answers with text, link and picture
 Admins can now pick, per question, how the player answers: free text, link, picture, or any mix. Each ticked box gets its own "correct answer" field, and the AI compares every part the player submits — including looking at their screenshot — into one score.
 Players see exactly the inputs the admin chose, can paste a screenshot with Ctrl+V, and their link/picture shows up in the review screen and in the admin grading queue.
@@ -1216,9 +1243,15 @@
 [agents-ai-scores] made a new "finish and send" feedback button, so admin wont be waitinf after every single feedback, to process, tehn send again.</t>
   </si>
   <si>
+    <t>10/08/2026 15:21:00</t>
+  </si>
+  <si>
     <t>updated the onex-academy website
 added new feature to uploade more than one images and links
 new feature to see all the prompts of the ai agents in the website, admin can edit  them all</t>
+  </si>
+  <si>
+    <t>21/08/2026 15:24:29</t>
   </si>
   <si>
     <t>[onex-academy]
@@ -1232,11 +1265,26 @@
 Added new “ai agents” section in ai-agents-scores website, so the admin can see all the ai agents prompt and edit however wants (created 2 workflows in n8n for that task, with two webhooks, POST to update(edit) the ai agents prompts, and GET for reading and showing the prompts in the website)</t>
   </si>
   <si>
+    <t>24/08/2026 15:57:23</t>
+  </si>
+  <si>
     <t>In ai-agents-scores project:
 Added Multi-criteria feedback display, editable ticket levels, per-criterion justification copy buttons.
 Fixed the blank dashboard that sometimes loaded zero tickets.
 Replaced the broken localStorage cache with IndexedDB and added automatic retries.
 Deleted unnecessary code, files, folders, variables, comments, functions, etc. Cleaned up the codebase.</t>
+  </si>
+  <si>
+    <t>25/08/2026 16:05:00</t>
+  </si>
+  <si>
+    <t>made new AI agentic workflow in n8n, with gets the new gmail messages, parses and gets the tracking codes(numbers) and order numbers(ids) and collecting that all into the special created google sheets, with the sender email, date-time, email from, email to, order id, tracking code, etc.. all the info has been storing and every 1 minute the workflow is being triggered and updating the google sheets list</t>
+  </si>
+  <si>
+    <t>26/08/2026 14:57:29</t>
+  </si>
+  <si>
+    <t>updated the ai agentic n8n workflow of the ONEX's Buy for me services automation in the gmail about the tracking code and order id/number</t>
   </si>
 </sst>
 </file>
@@ -1272,12 +1320,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1582,13 +1627,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B185"/>
+  <dimension ref="A1:B187"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
     <col min="2" max="2" width="100" style="1" customWidth="1"/>
-    <col min="3" max="17" width="8.88671875" style="1" customWidth="1"/>
-    <col min="18" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="19" width="8.88671875" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2696,379 +2741,395 @@
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A139" s="2">
-        <v>46196.602083333331</v>
+      <c r="A139" s="1" t="s">
+        <v>275</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A140" s="2">
-        <v>46197.602083333331</v>
+      <c r="A140" s="1" t="s">
+        <v>277</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A153" s="2">
-        <v>46213.625949074078</v>
+      <c r="A153" s="1" t="s">
+        <v>303</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="157" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" s="2">
-        <v>46219.619687500002</v>
+      <c r="A157" s="1" t="s">
+        <v>311</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A158" s="2">
-        <v>46220.619687500002</v>
+      <c r="A158" s="1" t="s">
+        <v>313</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="159" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="160" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
     </row>
     <row r="161" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="165" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="167" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
     <row r="168" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A168" s="2">
-        <v>46233.606053240743</v>
+      <c r="A168" s="1" t="s">
+        <v>333</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="171" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
     </row>
     <row r="173" spans="1:2" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="174" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
     </row>
     <row r="175" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="176" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A176" s="2">
-        <v>46245.666377314818</v>
+      <c r="A176" s="1" t="s">
+        <v>348</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
     </row>
     <row r="177" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A177" s="2">
-        <v>46246.666666666657</v>
+      <c r="A177" s="1" t="s">
+        <v>350</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
     </row>
     <row r="178" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="179" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="180" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" ht="409.6" x14ac:dyDescent="0.3">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" ht="403.2" x14ac:dyDescent="0.3">
-      <c r="A182" s="2">
-        <v>46253.63958333333</v>
+        <v>357</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" ht="403.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="1" t="s">
+        <v>358</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A183" s="2">
-        <v>46244.63958333333</v>
+        <v>359</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="1" t="s">
+        <v>360</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A184" s="2">
-        <v>46255.642002314817</v>
+        <v>361</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" ht="244.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="1" t="s">
+        <v>362</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" ht="72" x14ac:dyDescent="0.3">
-      <c r="A185" s="2">
-        <v>46258.664849537039</v>
+        <v>363</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" ht="72" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A185" s="1" t="s">
+        <v>364</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>353</v>
+        <v>365</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A186" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A187" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B187" s="1" t="s">
+        <v>369</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated the system and the saving style
</commit_message>
<xml_diff>
--- a/task_reports.xlsx
+++ b/task_reports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\semyONEX\semyon-not-work-lol\AI_ML_programmming\self_created_projects\task-report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3C2B57-8F7F-42A6-AF91-20B45F1F7C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EDF0A5-B1A2-4456-8E14-541562DF05D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-10980" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reports" sheetId="1" r:id="rId1"/>
@@ -1639,9 +1639,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100" style="1" customWidth="1"/>
-    <col min="3" max="20" width="8.88671875" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="203.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="21" width="8.88671875" style="1" customWidth="1"/>
+    <col min="22" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -3140,7 +3140,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="188" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:2" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>370</v>
       </c>

</xml_diff>

<commit_message>
nice update, now the same day's tasks are being merget into the same cell and that tasks date time is being updated
</commit_message>
<xml_diff>
--- a/task_reports.xlsx
+++ b/task_reports.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-10980" windowWidth="29040" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Reports" sheetId="1" state="visible" r:id="rId1"/>
@@ -421,13 +421,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B189"/>
+  <dimension ref="A1:B194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="25" customWidth="1" style="1" min="1" max="1"/>
     <col width="203.77734375" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
-    <col width="8.88671875" customWidth="1" style="1" min="3" max="22"/>
-    <col width="8.88671875" customWidth="1" style="1" min="23" max="16384"/>
+    <col width="8.88671875" customWidth="1" style="1" min="3" max="23"/>
+    <col width="8.88671875" customWidth="1" style="1" min="24" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
@@ -450,7 +450,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Created ai agentic workflow with the necessary main algorithm with right logic which gets bad estimation and the prompt of an ai agent: improves prompt, validates it(if still invalid updates prompt again, then validates) then rewriting the prompt.</t>
+          <t>Created an AI agentic workflow with the main algorithm and correct logic: it takes a poor estimation together with an AI agent's prompt, improves the prompt, validates it (if it is still invalid, updates the prompt again and re-validates), and then rewrites the prompt.</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>I've created local Docker containers to run n8n, and added a new Telegram bot feature to the self-improving prompt workflow. Now, nice notifications occur when the prompt is updated, and the prompt is sent as a text file by the bot to a specific user.</t>
+          <t>Created local Docker containers to run n8n, and added a new Telegram bot feature to the self-improving prompt workflow. Notifications are now sent when the prompt is updated, and the prompt is delivered as a text file by the bot to a specific user.</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>I have created a new n8n data table for the ticket analyzer agent's prompt, so that the summary generator and estimator workflow, and the self-improving prompt updater workflow, will access the same prompt, and updates will work on both workflows successfully.</t>
+          <t>Created a new n8n data table for the ticket analyzer agent's prompt, so that both the summary generator and estimator workflow and the self-improving prompt updater workflow access the same prompt, and updates apply to both workflows successfully.</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>I have updated the workflow of the Ticket Analyzer AI agent. It now sends `chat_history` and `ticket_id` values to Supabase, as intended. I have also worked on the self-improving system, which will be completed tomorrow.</t>
+          <t>Updated the Ticket Analyzer AI agent's workflow. It now sends the chat_history and ticket_id values to Supabase, as intended. Also continued working on the self-improving system, which will be completed tomorrow.</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>I have finished the self-improving workflow, so it now works with the production URL. I fixed the bug in the ticket analyzer agent workflow, and I've started researching suitable, high-quality Armenian speech-to-text models (like 11labs, wav.am, etc.). I've also begun creating an Armenian speech-to-text workflow to analyze and handle customer support calls.</t>
+          <t>Finished the self-improving workflow, so it now works with the production URL. Fixed the bug in the ticket analyzer agent's workflow, and started researching suitable, high-quality Armenian speech-to-text models (ElevenLabs, WAV.am, etc.). Also began creating an Armenian speech-to-text workflow to analyze and handle customer support calls.</t>
         </is>
       </c>
     </row>
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A new workflow has been created that retrieves an audio file, sends it to WAV.am via an HTTP request to obtain the translation, receives it back, and then structures the call transcription as a conversation between a customer and a call support agent. It works well, and the aim is to replicate this for chat support to enable analysis with the same model.</t>
+          <t>Created a new workflow that retrieves an audio file, sends it to WAV.am via an HTTP request to obtain the transcription, receives it back, and then structures the call transcription as a conversation between a customer and a call support agent. It works well, and the aim is to replicate it for chat support so that the same model can be used for analysis.</t>
         </is>
       </c>
     </row>
@@ -522,7 +522,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>I improved the speech-to-text n8n workflow, created and enhanced a new prompt for the extractor agent (the AI agent that structures call conversations), and also conducted some tests of Armenian speech-to-text to benchmark the corresponding speech-to-text model.</t>
+          <t>Improved the speech-to-text n8n workflow, created and enhanced a new prompt for the extractor agent (the AI agent that structures call conversations), and ran tests of Armenian speech-to-text in order to benchmark the corresponding model.</t>
         </is>
       </c>
     </row>
@@ -534,10 +534,10 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>1. I have created a workflow that takes real support call audio (MP3), extracts the conversational text (structured as JSON, the same way as the support chat format), and then provides this to the next agent. This agent is the same one who analyzes support chat tickets. The conversation is processed identically to how the 'ticket analyzer' handles support chat conversations. The workflow is the same as the chat analyzer, and it will ultimately add a new column to Supabase(in the future) with the same structure as it does in the chat ticket analyzing workflow. The only difference is in the first stage, where the voice MP3 file is converted to text.
-2. I have also developed test cases and analyzed the results from the real call speech-to-text WAV.am model. I have compiled a 'models-mistakes' txt document detailing the model's errors that I have observed. This document will be instrumental in building a robust AI agent system prompt, ensuring the AI agent is aware of potential speech model inaccuracies and can correct them. I have analyzed 18 calls and have 16 more calls that I have yet to benchmark. I have requested additional calls(right now I have 34 call mp3 files).
-*All the tests i have done with WAV.am model, which handles the default mp3 format of the call
-3. Additionally, I will begin researching other Armenian speech-to-text models (such as ElevenLabs, etc.) to determine the highest quality model for our support call extracting task.</t>
+          <t>1. Created a workflow that takes real support call audio (MP3), extracts the conversational text (structured as JSON, in the same format as support chats), and passes it to the next agent — the same agent that analyzes support chat tickets. The conversation is processed identically to the way the "ticket analyzer" handles support chat conversations. The workflow mirrors the chat analyzer and will eventually add a new column to Supabase with the same structure as in the chat ticket analyzing workflow. The only difference is the first stage, where the MP3 voice file is converted to text.
+2. Developed test cases and analyzed the results of the WAV.am speech-to-text model on real calls. Compiled a "model mistakes" text document detailing the errors observed. This document will be instrumental in building a robust AI agent system prompt, ensuring that the agent is aware of potential speech model inaccuracies and can correct them. Analyzed 18 calls, with 16 more still to benchmark, and requested additional calls (currently there are 34 call MP3 files).
+Note: all tests were performed with the WAV.am model, which handles the default MP3 format of the calls.
+3. Will also begin researching other Armenian speech-to-text models (such as ElevenLabs) in order to determine the highest-quality model for the support call extraction task.</t>
         </is>
       </c>
     </row>
@@ -549,8 +549,8 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Researched and became familiar with the Ladesk system, created a new pipeline for audio files to be sent to n8n for processing. The system now automatically sends every resolved call ticket to n8n, where the corresponding call audio file is converted to Armenian text and then into a structured JSON message, similar to the support chat ticket.
-Additionally, created a new rule in Ladesk to send the call ticket JSON data to n8n, utilizing the already established n8n API within Ladesk.</t>
+          <t>Researched and became familiar with the Ladesk system, and created a new pipeline for sending audio files to n8n for processing. The system now automatically sends every resolved call ticket to n8n, where the corresponding call audio file is converted into Armenian text and then into a structured JSON message, similar to a support chat ticket.
+Also created a new rule in Ladesk to send call ticket JSON data to n8n, using the n8n API already configured in Ladesk.</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>I have resolved the issue of multiple calls within a single ticket in the n8n workflow and have corrected the Supabase row adding node.</t>
+          <t>Resolved the issue of multiple calls within a single ticket in the n8n workflow, and corrected the Supabase row-adding node.</t>
         </is>
       </c>
     </row>
@@ -574,9 +574,9 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>I found a way to estimate call duration in n8n, based on the audio file’s byte size, header length, and similar nuances. This approach results in an approximate ±1–12 seconds deviation from the actual call duration. In my assessment, this accuracy is acceptable and can be used.
-I calculated that, statistically, approximately 600–900 calls are resolved per day. At a later stage, I will calculate the total aggregated call duration per day (or per month) in order to estimate the overall cost, for example when using WAV.am.
-I benchmarked ~24 calls and documented the observed errors.</t>
+          <t>Found a way to estimate call duration in n8n based on the audio file's byte size, header length, and similar details. This approach produces an approximate deviation of ±1–12 seconds from the actual call duration, and in my assessment this accuracy is acceptable and can be used.
+Calculated that, statistically, approximately 600–900 calls are resolved per day. At a later stage, will calculate the total aggregated call duration per day (or per month) in order to estimate the overall cost, for example when using WAV.am.
+Benchmarked around 24 calls and documented the observed errors.</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>I made a summary of the speech-to-text model's mistakes. Considering this, I performed prompt engineering and improved the model's call conversation extraction. Now, the model extracts better call conversation quality, which is beneficial for the next step: an Analyzer AI agent to analyze and make high-quality estimations regarding the quality assurance of the call support agent.</t>
+          <t>Summarized the speech-to-text model's mistakes. Based on that, performed prompt engineering and improved the model's extraction of call conversations. The model now extracts call conversations of better quality, which benefits the next step: an analyzer AI agent that produces high-quality estimations for the quality assurance of call support agents.</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Improved chat and call ticket analyzer workflows. They are now adding new 'chat' or 'call' statuses in the newly added status column in Supabase. A lot of tests were also performed, and the call extractor agent's prompt was improved.</t>
+          <t>Improved the chat and call ticket analyzer workflows. They now add a "chat" or "call" status in the newly added status column in Supabase. Also ran a large number of tests and improved the call extractor agent's prompt.</t>
         </is>
       </c>
     </row>
@@ -612,8 +612,8 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>I tested and improved(cosidering its mistakes) the prompt for the support call extractor agent, and it works well. I have also created and implemented new methods for obtaining number of currently active tickets(call tickets) and resolved(today's) ticket numbers using n8n's HTTP request node and code node.
-Furthermore, I have investigated LiveAgent's API documentation to implement all of these features.</t>
+          <t>Tested and improved the support call extractor agent's prompt (taking its mistakes into account), and it now works well. Also created and implemented new methods for obtaining the number of currently active call tickets and the number of tickets resolved today, using n8n's HTTP Request and Code nodes.
+In addition, investigated LiveAgent's API documentation in order to implement all of these features.</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>I have created a new node chain in the n8n workflow to retrieve today's number of calls in the queue and the number of missed callbacks. I have also investigated the GET/POST /ticket and GET /calls endpoints from LiveAgent API Documentation to implement this.</t>
+          <t>Created a new node chain in the n8n workflow to retrieve today's number of calls in the queue and the number of missed callbacks. Also investigated the GET/POST /ticket and GET /calls endpoints in the LiveAgent API documentation in order to implement this.</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>I have improved the overall performance and accuracy of the live call statistics display(In an n8n workflow, using LiveAgent API v3 calls, HTTP requests which are pipelined between n8n and Ladesk.) for the further statistics table. I have also made perecise calculations and display of today's call ticket statistics, including calls per hour, one call every X minutes, number of ongoing calls, number of calls in queue, number of resolved calls today, number of missed calls today, and number of calls that were missed and have been called back, among others.</t>
+          <t>Improved the overall performance and accuracy of the live call statistics display (in an n8n workflow, using LiveAgent API v3 calls and HTTP requests pipelined between n8n and Ladesk) for the upcoming statistics table. Also implemented precise calculation and display of today's call ticket statistics, including calls per hour, one call every X minutes, the number of ongoing calls, the number of calls in the queue, the number of calls resolved today, the number of calls missed today, and the number of missed calls that have been called back, among others.</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>I replaced the standard 'click to trigger' node with a webhook, including its URL in 'call statistic sender' n8n workflow. This will ensure that call statistics are sent to Lovable every x minutes using that webhook URL. Additionally, I've added new statistics: 'avg. call duration' and 'total duration of calls (today's all calls summary)'. Made all that statistics to be nice structured to get and deploy easly.</t>
+          <t>Replaced the standard "click to trigger" node with a webhook, including its URL, in the "call statistics sender" n8n workflow. This ensures that call statistics are sent to Lovable every X minutes through that webhook URL. Also added new statistics — average call duration and total call duration (a summary of all of today's calls) — and structured all of these statistics so that they can be retrieved and deployed easily.</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>I have created new statistics for the call center statistics n8n workflow, including the busiest call agent, call duration percentages, and distributions of other insightful statistical values. I have also received new tasks concerning chat agent performance and other chat statistics.</t>
+          <t>Created new statistics for the call center statistics n8n workflow, including the busiest call agent, call duration percentages, and the distribution of other insightful statistical values. Also received new tasks concerning chat agent performance and other chat statistics.</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>I created and improved an n8n workflow that now sends new chat statistics (number of busy agents in chat and their names in a list, number of chats in queue) via HTTP request and Webhook. I also changed the 'calls per x minute' to 'calls per x second', and received new tasks regarding call summary classification and WAV.am score spending statistics on calls, as well as a task concerning caller number fixing.</t>
+          <t>Created and improved an n8n workflow that now sends new chat statistics (the number of agents busy in chat and their names as a list, and the number of chats in the queue) via HTTP request and webhook. Also changed "calls per X minutes" to "calls per X seconds", and received new tasks regarding call summary classification, WAV.am score spending statistics for calls, and caller number fixing.</t>
         </is>
       </c>
     </row>
@@ -685,8 +685,8 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>I created new variable and calculated how many score costs an audioto transcribe using WAV.am, and also created new variable which gets the customers phone number and fixed both variables.
-I am working on creating new AI Agent, who will get the chat or call(text version), tags and make summary classification(it will choose one of the fixed summary classifications or if the input doesn't correspond to any it will suggest one)</t>
+          <t>Created a new variable and calculated the score cost of transcribing an audio file with WAV.am, and created another new variable that retrieves the customer's phone number; fixed both variables.
+Currently working on a new AI agent that will take the chat or call (text version) together with the tags and produce a summary classification (it will choose one of the fixed summary classifications or, if the input does not correspond to any of them, suggest a new one).</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>I fixed and made up to deploy state the statistics numbers extracting from tickets, in particular extracting customer_number from ticket, cost of the support call audio transcribe(WAV.am score), and trendng_summary which first classifies the arrived ticket(chat/call history), so the AI Scoring system(or the new one, regarding only support calls) which will store the counts of each category and show the Most trending topics of the &lt;period of time&gt; statistics and getting the count from http request node which I have created to make that as an end point.</t>
+          <t>Fixed and brought to a deployable state the extraction of statistical figures from tickets — in particular the customer number, the cost of transcribing the support call audio (WAV.am score), and the trending summary, which first classifies the incoming ticket (chat or call history) so that the AI scoring system (or the new one, covering support calls only) can store the counts for each category and display the most trending topics for a given period. The counts are retrieved through the HTTP Request node that I created as an endpoint.</t>
         </is>
       </c>
     </row>
@@ -710,9 +710,9 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>I created new some data tables, one for call/chat support centre's corresponding day's statistics, the other for history of each day(every day 23:53 it will be saved and the numbers will be resetted to 0, for the next day's statistics).
-I have inproved statistical choice maker(aka summarization alayst) AI Agent't prompt, improved and developed its workflows, to work correctly in call and chat support workflows separately(added new nodes to change/insert/get/write in n8n data tables, etc. to implement all the logic), made tests to fix errors and bugs in the mentioned workflows and to inhance AI Agents prompt(more stable and robust).
-I have also created new workflow which resetes all the statisticall trending topics values to 0 and saves the previous day's statistics in the statistical history data table, ensuring no data will be lost.</t>
+          <t>Created several new data tables: one for the call and chat support center's statistics for the current day, and another for the history of each day (every day at 23:53 the figures are saved and reset to 0, ready for the next day's statistics).
+Improved the prompt of the statistical choice maker (the summarization analyst) AI agent, and improved and developed its workflows so that they work correctly in the call and chat support workflows separately (added new nodes to change, insert, get and write in n8n data tables, and so on, in order to implement all the logic). Also ran tests to fix errors and bugs in these workflows and to make the AI agent's prompt more stable and robust.
+In addition, created a new workflow that resets all statistical trending topic values to 0 and saves the previous day's statistics in the statistics history data table, ensuring that no data is lost.</t>
         </is>
       </c>
     </row>
@@ -724,8 +724,8 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>I created new workflow to trigger and get the trending topics using Webhook, so we can connect that with the AI Scoring site.
-made changing in the LiveAgent and Call ticket analyzer workflows, now the system checks, if the suggestion exists, then adds that suggestion to the new created data table in the n8n, if there is no sugesstion and classifier AI agent mades decision to classify it with one of the mentioned trending list, then the workflow continues in a natural way(the old way), this ensures of workflow stopping or errors caused by the suggestion existance and trending topic emptiness.</t>
+          <t>Created a new workflow that is triggered by a webhook and returns the trending topics, so that it can be connected to the AI Scoring site.
+Made changes to the LiveAgent and call ticket analyzer workflows: the system now checks whether a suggestion exists and, if it does, adds that suggestion to the newly created n8n data table; if there is no suggestion and the classifier AI agent decides to classify the ticket with one of the listed trending topics, the workflow continues in the usual way. This prevents the workflow from stopping or throwing errors caused by the existence of a suggestion or by an empty trending topic.</t>
         </is>
       </c>
     </row>
@@ -737,8 +737,8 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>I updated the list of trending topics for the classifier agent prompt; I also improved the workflow, making it more robust, and performed some prompt engineering on our AI summary classifier agent. 
-Got new tasks regarding the support agents' quality management AI estimation tools, as well as AI video-making prompt engineering tasks.</t>
+          <t>Updated the list of trending topics in the classifier agent's prompt, improved the workflow to make it more robust, and performed prompt engineering on the AI summary classifier agent.
+Also received new tasks regarding the support agents' quality management AI estimation tools, as well as AI video-making prompt engineering tasks.</t>
         </is>
       </c>
     </row>
@@ -750,8 +750,8 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>I worked on generating videos for ONEX's Support Call Center's tutorial phase, which will be used to train new agents to statr working. I created some examples and discussed the results, which led to new tasks.
-I checked n8n's 'other topics' data table to identify topics that the AI Classifier agent couldn't categorize, which means that it suggests adding them to the fixed list.</t>
+          <t>Worked on generating videos for the tutorial phase of ONEX's support call center, which will be used to train new agents. Created several examples and discussed the results, which led to new tasks.
+Also checked n8n's "other topics" data table in order to identify topics that the AI classifier agent could not categorize, which means that it suggests adding them to the fixed list.</t>
         </is>
       </c>
     </row>
@@ -763,8 +763,8 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>I updated the prompt of the AI Classifier agent, adding a few new trending topics based on the AI's suggestions.
-I also updated and improved its workflow, which now sends the corresponding ticket ID of the newly suggested topic so I can know what kind of topic to add to the fixed list.</t>
+          <t>Updated the AI classifier agent's prompt, adding a few new trending topics based on the AI's suggestions.
+Also updated and improved its workflow, which now sends the corresponding ticket ID for each newly suggested topic, so that I can see what kind of topic should be added to the fixed list.</t>
         </is>
       </c>
     </row>
@@ -776,8 +776,8 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>I received the necessary files containing November, December, and January data for support call center agents' quality (chat and call). I started working on the statistics drawer and the calculator workflow (or code).
-Also, I checked the 'other trending topics' data table in n8n to create new trending topics, so the AI Classifier agent should have that new option as well.</t>
+          <t>Received the necessary files containing the November, December and January data on support call center agents' quality (chat and call), and started working on the statistics drawer and the calculator workflow (or code).
+Also checked the "other trending topics" data table in n8n in order to create new trending topics, so that the AI classifier agent has these new options as well.</t>
         </is>
       </c>
     </row>
@@ -789,8 +789,8 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>I created a code that will parse the received Excel file into a structured CSV, which will allow me to plot and draw some statistical and other graphs to visualize and analyze the specific agent's statistics, performance, etc.
-I also made a separate code and conducted tests of plotting the statistics graphs.</t>
+          <t>Created code that parses the received Excel file into a structured CSV, which makes it possible to plot statistical and other graphs in order to visualize and analyze a specific agent's statistics, performance, and so on.
+Also wrote separate code and ran tests for plotting the statistics graphs.</t>
         </is>
       </c>
     </row>
@@ -802,8 +802,8 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>I created a new Streamlit project which allows comparing and selecting the necessary agents to view and compare their statistics.
-I also wrote code that retrieves the Excel data file and converts it into a fully structured and functional CSV file, with well-structured and clean data.</t>
+          <t>Created a new Streamlit project that makes it possible to select and compare the required agents in order to view their statistics.
+Also wrote code that reads the Excel data file and converts it into a fully structured and functional CSV file with clean, well-structured data.</t>
         </is>
       </c>
     </row>
@@ -815,8 +815,8 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Developed a functional web platform that allows users to upload structured data files and receive automated statistical analysis and performance insights. The current version supports data ingestion and visualization, with additional improvements and refinements planned.
-In parallel, work has begun on designing and implementing new AI agents aimed at evaluating service performance quality. These agents will analyze operational data and generate assessments based on predefined evaluation criteria. The focus is on building an automated, scalable system capable of consistent and objective performance analysis.</t>
+          <t>Developed a functional web platform that allows users to upload structured data files and receive automated statistical analysis and performance insights. The current version supports data ingestion and visualization, and further improvements and refinements are planned.
+In parallel, began designing and implementing new AI agents intended to evaluate service performance quality. These agents will analyze operational data and generate assessments based on predefined evaluation criteria. The focus is on building an automated, scalable system capable of consistent and objective performance analysis.</t>
         </is>
       </c>
     </row>
@@ -828,8 +828,8 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>I made new architectures for the 'Liveagent resolved tickets' and 'call analyzer' n8n AI Agentic workflows. The classifying AI agent in these workflows gets the allowed trending topics list from the data table, making it highly dynamic and flexible. Therefore, if we add new trending topics based on the AI Agent's suggestions in the data table, the list should be automatically updated in the prompt of the AI Classifier agent in both n8n workflows.
-Also, I extracted criteria from the customer support control call/chat agents statistics Excel file and prepared to create AI agents to perform the same rating for further statistics.</t>
+          <t>Created new architectures for the "LiveAgent resolved tickets" and "call analyzer" n8n AI agentic workflows. The classifying AI agent in these workflows now takes the list of allowed trending topics from the data table, which makes it highly dynamic and flexible. As a result, when new trending topics are added to the data table based on the AI agent's suggestions, the list is updated automatically in the AI classifier agent's prompt in both n8n workflows.
+Also extracted the criteria from the customer support control call and chat agent statistics Excel file, and prepared to create AI agents that will perform the same rating for further statistics.</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Created two new n8n AI agents: an analyzer and a grader. The analyzer AI agent analyzes resolved tickets and passes that analysis to the grader AI agent, which then assigns grades and ratings for every provided criterion, along with comments for each. All results are added to a nicely structured Google Sheet. Also, I improved the agents' prompts and generated valid and robust results. I've added all these agents and their parser code nodes into the Chat Analyzer n8n AI agentic workflow, and it works well.</t>
+          <t>Created two new n8n AI agents: an analyzer and a grader. The analyzer agent analyzes resolved tickets and passes its analysis to the grader agent, which then assigns grades and ratings for every provided criterion, along with a comment for each. All results are added to a neatly structured Google Sheet. Also improved the agents' prompts and generated valid, robust results, and added both agents and their parser code nodes to the chat analyzer n8n AI agentic workflow, where they work well.</t>
         </is>
       </c>
     </row>
@@ -853,8 +853,8 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Updated prompts for the grader and analyzer AI agents (based on the discussion with the quality support specialist).
-Added a new function that adds the name of a support service agent to the Google Sheet's corresponding data point.</t>
+          <t>Updated the prompts of the grader and analyzer AI agents (based on the discussion with the quality support specialist).
+Added a new function that writes the name of the support service agent to the corresponding data point in the Google Sheet.</t>
         </is>
       </c>
     </row>
@@ -866,10 +866,10 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Fixed error in 'google sheets' node.
-Updated Analyzer and Grader AI Agents system prompts and Google Sheet node's structure.
-Updateed lovable web app to parse and calculate, handle the right data.
-The structure of the results of the google sheet file from the new analyzer-grader n8n AI agents has been changed, now yielding more effective and chat-related grades and corresponding comments.</t>
+          <t>Fixed an error in the Google Sheets node.
+Updated the system prompts of the analyzer and grader AI agents and the structure of the Google Sheets node.
+Updated the Lovable web app so that it parses, calculates and handles the correct data.
+Changed the structure of the results in the Google Sheet produced by the new analyzer-grader n8n AI agents, which now yield more effective, chat-related grades with corresponding comments.</t>
         </is>
       </c>
     </row>
@@ -881,10 +881,10 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Made improvements to the AI call center agents' statistics and ratings website, creating a new method for data handling and several new statistical features and visualizations (significantly updating the UI, frontend structure, and data handling).
-Created a new n8n AI workflow to send data to this website, which visualizes all of it nicely and robustly.
-I also generated an AI video and made some nice improvements to the video editing.
-Got new tasks for further projects.</t>
+          <t>Improved the AI call center agents' statistics and ratings website, creating a new data handling method and several new statistical features and visualizations (which significantly updated the UI, the frontend structure and the data handling).
+Created a new n8n AI workflow that sends data to this website, which visualizes all of it neatly and robustly.
+Also generated an AI video and made several improvements to the video editing.
+Received new tasks for further projects.</t>
         </is>
       </c>
     </row>
@@ -896,8 +896,8 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>We performed a massive upgrade on the agent's AI scoring web interface.
-New features were added, and the colors were made nicer and richer to correspond with the ONEX brand.</t>
+          <t>Performed a major upgrade of the agents' AI scoring web interface.
+Added new features and made the colors nicer and richer, so that they correspond to the ONEX brand.</t>
         </is>
       </c>
     </row>
@@ -909,15 +909,15 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Core Features &amp; Logic
-Ticket Simulation: Implemented logic for automatic ticket generation (intervals, hourly/weekly patterns) and peak hour analytics.
-n8n Integration: Connected Agent prompts to n8n data tables to enable dynamic, self-improving workflows.
-UI &amp; Visualization
-Smart Dashboard: Redesigned KPI cards ("number blocks") with a cleaner layout and dynamic color coding.
-Enhanced Charts: Added smart tooltips to graphs that instantly highlight the highest scores and top agents.
-Agent Comparison: Improved the readability of comparison blocks while preserving detailed hover interactions.
-General Updates
-Branding: Updated the sidebar menu, copyright text, and increased the ONEX logo size for better visibility.</t>
+          <t>Core features and logic
+Implemented ticket simulation logic for automatic ticket generation (intervals, hourly and weekly patterns) and peak hour analytics.
+Connected the agent prompts to n8n data tables in order to enable dynamic, self-improving workflows.
+UI and visualization
+Redesigned the smart dashboard KPI cards ("number blocks") with a cleaner layout and dynamic color coding.
+Enhanced the charts by adding smart tooltips that instantly highlight the highest scores and the top agents.
+Improved the readability of the agent comparison blocks while preserving the detailed hover interactions.
+General updates
+Updated the sidebar menu and the copyright text, and increased the size of the ONEX logo for better visibility.</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Implemented advanced Tickets filtering with three case-insensitive searches (agent, ticket number, conversation) plus multi-select LEVEL 1/2/3 filtering, all combined with date/agent filters in one pipeline. Added conversation search coverage for both comments and chat history, and renamed “Raw Data” to “Tickets.” Secured the app with login/logout, protected routes, and basic failed-attempt lockout/session handling, then verified with successful tests/build.</t>
+          <t>Implemented advanced ticket filtering with three case-insensitive searches (agent, ticket number and conversation), plus multi-select LEVEL 1/2/3 filtering, all combined with the date and agent filters in a single pipeline. Added conversation search coverage for both comments and chat history, and renamed "Raw Data" to "Tickets". Secured the app with login and logout, protected routes, and basic failed-attempt lockout and session handling, then verified everything with successful tests and a successful build.</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Add new evaluation criteria: Chat start (yes/no), Need identified (yes/no), if need exists but not asked → bad (1/0), proper handling → good (5), and empathy emoji/expression (yes/no).
-Display criteria grouped together in the Tickets section and apply fixed weights; if one is missing or null, redistribute its weight across the remaining criteria.
-Remove Hourly Activity, Weekly Activity, and Satisfaction Trends.
-In Score Distribution, enable clicking a score (e.g., 5) to open the full list of matching tickets with the same functionality as the Tickets section.
-In Skill Group Overview, group skills according to Anna’s provided structure and display them under the triangle section.
-At chat end, check whether the customer closed the chat and score accordingly; also ensure graph colors are максимально distinct.</t>
+          <t>Added new evaluation criteria: chat start (yes/no) and need identified (yes/no); if a need exists but is not asked about → bad (1/0), proper handling → good (5), plus an empathy emoji or expression criterion (yes/no).
+Displayed the criteria grouped together in the Tickets section and applied fixed weights; if one of them is missing or null, its weight is redistributed across the remaining criteria.
+Removed Hourly Activity, Weekly Activity and Satisfaction Trends.
+Made the scores in Score Distribution clickable, so that clicking a score (for example 5) opens the full list of matching tickets with the same functionality as the Tickets section.
+Grouped the skills in Skill Group Overview according to the structure provided by Anna and displayed them under the triangle section.
+Added a check at the end of a chat for whether the customer closed the chat and scored it accordingly, and also made the graph colors as distinct as possible.</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Updated the AI agent scoring UI: donut chart colors were refined (Excellent/Good greens), and cluster weight editing was redesigned to be per-cluster via an Edit Weights modal (no always-open fields). Weights are now edited as percentages, require a strict 100% total per cluster, and can be applied either to the current ticket or to all tickets. Added "today", "yesterday", "last week", "last month", and "reset" buttons to the date-time filtering section. Also started creating new internet searching AI workflow for FPL Captain web site.</t>
+          <t>Updated the AI agent scoring UI: refined the donut chart colors (greens for Excellent and Good) and redesigned cluster weight editing so that it is done per cluster through an Edit Weights modal instead of always-open fields. Weights are now edited as percentages, require a strict total of 100% per cluster, and can be applied either to the current ticket or to all tickets. Added "Today", "Yesterday", "Last week", "Last month" and "Reset" buttons to the date and time filtering section. Also started creating a new internet-searching AI workflow for the FPL Captain website.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implemented a per-agent ticket popup from Agent Details, so every card can open all tickets for that selected agent. </t>
+          <t>Implemented a per-agent ticket popup in Agent Details, so that every card can open all of the tickets for the selected agent.</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Finished AI Article Maker for FPL Capitain, improved AI agents system prompt and image generator AI Agents prompt. Had long discussion about future AI projects with the CTO.</t>
+          <t>Finished the AI Article Maker for FPL Captain, and improved the AI agents' system prompt and the image generator AI agent's prompt. Also had a long discussion with the CTO about future AI projects.</t>
         </is>
       </c>
     </row>
@@ -994,8 +994,8 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Updated the list of trending topics in the n8n data tables, also updated the prompt for corresponding agent, so it will consider(and cover from now on) that topics also.
-Updated the AI Agents Scoring web sites sorting and filtering, searching algorithms.</t>
+          <t>Updated the list of trending topics in the n8n data tables, and updated the corresponding agent's prompt so that it now takes these topics into account as well.
+Also updated the sorting, filtering and searching algorithms of the AI Agents Scoring website.</t>
         </is>
       </c>
     </row>
@@ -1007,8 +1007,8 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>updated ai image generator prompt so it will generate the title text of the article at the bottom-left part of the image
-Updated the whole AI article maker n8n workflow the ai article maker agent’s prompt and pervious articles(in prompt) are being got from the n8n data tables.</t>
+          <t>Updated the AI image generator prompt so that it generates the article's title text in the bottom-left part of the image.
+Updated the entire AI article maker n8n workflow: the article maker agent's prompt and the previous articles used in the prompt are now retrieved from the n8n data tables.</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Made the prototype of the Options Summarizer and compared AI n8n workflow. Improved the agent's prompt. Made the output valid CSV.</t>
+          <t>Created the prototype of the Options Summarizer and comparison AI n8n workflow. Improved the agent's prompt and made the output valid CSV.</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Updated n8n workflow of AI option summarizer. Trying to make that to handle as many documents as you send it using webhook.</t>
+          <t>Updated the n8n workflow of the AI option summarizer. Currently working on making it handle as many documents as are sent to it through the webhook.</t>
         </is>
       </c>
     </row>
@@ -1044,9 +1044,9 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Made updates in the AI option summarizer n8n workflow:
-Updated the prompt of the AI summarizer agent, so now the workflow outputs JSON (nicely structured) instead of CSV.
-Made improvements in the workflow to parse, regex, and make valid JSON out of the AI agent's output.</t>
+          <t>Made updates to the AI option summarizer n8n workflow:
+Updated the AI summarizer agent's prompt, so the workflow now outputs neatly structured JSON instead of CSV.
+Improved the workflow so that it parses the AI agent's output with regex and produces valid JSON.</t>
         </is>
       </c>
     </row>
@@ -1058,8 +1058,8 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Made a new n8n workflow for a self-improving agents system for an AI agents score site.
-Made an n8n option summarizer workflow in a ready-to-test state, which includes a ready webhook URL, working tested AI agents, and output processing parsing and sending back.</t>
+          <t>Created a new n8n workflow for a self-improving agent system for the AI agents score site.
+Brought the n8n option summarizer workflow to a ready-to-test state, including a ready webhook URL, tested and working AI agents, and output processing, parsing and sending back.</t>
         </is>
       </c>
     </row>
@@ -1071,8 +1071,8 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Created a new 'bad' button for feedback in the AI agents scoring site. Using that button and writing the reason, the prompt should be updated, and the AI agent should be upgraded and trained by us.
-Also starting work on n8n AI agent's prompt self-improving workflow for that button to handle and work.</t>
+          <t>Created a new "bad" feedback button on the AI agents scoring site. When the button is used and a reason is written, the prompt is updated so that the AI agent can be upgraded and trained.
+Also started working on the n8n AI agent prompt self-improving workflow that handles this button.</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Improved n8n AI self-improving prompt updating and validating testing workflow to get the right prompts. Also started working on getting the right necessary ticket metadata to process and use in the n8n workflow.</t>
+          <t>Improved the n8n AI self-improving workflow for prompt updating, validating and testing, in order to obtain the correct prompts. Also started working on retrieving the necessary ticket metadata to process and use in the n8n workflow.</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Started working on the Dropify project for Georgia, which includes an N8N workflow with AI, website parsing, and an AI agent that will get the specific product prices.</t>
+          <t>Started working on the Dropify project for Georgia, which includes an n8n workflow with AI, website parsing, and an AI agent that will retrieve specific product prices.</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Made some research regarding scraping sites for Dropify, its different ways, prices, etc.</t>
+          <t>Researched site scraping for Dropify, including the different approaches available, their prices, and so on.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>I made n8n self-improving AI workflow published, so it will get calls when inactive, and updated the website of AI agents score. So when clicking the new 'bad' button and writing the reason, the call should be sent to the n8n workflow. Made some tests, the workflow is in the testing state.</t>
+          <t>Published the n8n self-improving AI workflow, so that it receives calls while inactive, and updated the AI agents score website: clicking the new "bad" button and writing the reason now sends a call to the n8n workflow. Ran several tests; the workflow is in the testing state.</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Continued working on n8n AI self-improving workflow for AI Agents Score project, updated its prompt to correspond with the prompt updating, and in the right state.</t>
+          <t>Continued working on the n8n AI self-improving workflow for the AI Agents Score project, and updated its prompt so that it corresponds to the prompt updating logic and is in the correct state.</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Continued working on n8n self-improving AI workflow. Starting to add a new code node to parse messages in the right way from ticket data.</t>
+          <t>Continued working on the n8n self-improving AI workflow. Started adding a new code node to parse the messages from the ticket data correctly.</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Created new data table in n8n and started to connecting them to make right and correct pipelining for self-improving agents of AI agents' scoring (to update prompts correctly).</t>
+          <t>Created a new data table in n8n and started connecting the tables in order to build correct pipelining for the self-improving agents of the AI agents scoring project, so that the prompts are updated correctly.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>started working on new delivery data, to get coordinated from them and working on the future project about tracking delivers</t>
+          <t>Started working on the new delivery data in order to obtain coordinates from it, and began work on the future project for tracking deliveries.</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Crafted Website for Visualizing the Delivery Courier Data Points, and the Distance Between Them. Made Some Code to Parse and Pre-process the Data, to Extract Coordinates from Addresses, Etc.</t>
+          <t>Crafted a website for visualizing the delivery courier data points and the distances between them. Also wrote code to parse and pre-process the data and to extract coordinates from addresses.</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Researched updated data points of delivery courier data.</t>
+          <t>Researched the updated data points of the delivery courier data.</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Meet with the AI agents, score users, and inform them to use the newly created self-improving workflow trigger button, named 'Bad Response', to test it in further cases and make it ready for presentation and use.</t>
+          <t>Met with the AI agents score users and instructed them to use the newly created self-improving workflow trigger button, named "Bad Response", in order to test it in further cases and make it ready for presentation and use.</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Meet with Customer Support Quality Specialist and presented the new 'Send Feedback' button, to train AI agents to start giving correct estimations and grades.</t>
+          <t>Met with the Customer Support Quality Specialist and presented the new "Send Feedback" button, which is used to train the AI agents so that they start giving correct estimations and grades.</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Researched, deployed, and tested some Armenian STT models from GitHub to add them to our AI agents' score system. Also got feedback from the AI grader and analyzer agents' system from a quality control head. Made tasks from them to do in the future.</t>
+          <t>Researched, deployed and tested several Armenian speech-to-text models from GitHub, with a view to adding them to the AI agents score system. Also received feedback on the AI grader and analyzer agent system from the head of quality control, and turned that feedback into tasks for the future.</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Task Report. Reviewed Agents AI scores requirements from the chat with Head of Quality Control and developed the feedback form tasks. Implemented a new feature allowing users to submit feedback for Grader and Analyzer agents multiple times per ticket. Updated all criteria names to align exactly with the excel files for consistency.</t>
+          <t>Reviewed the AI agents score requirements from the chat with the Head of Quality Control and developed the feedback form tasks. Implemented a new feature that allows users to submit feedback for the grader and analyzer agents several times per ticket. Updated all criteria names so that they align exactly with the Excel files, for consistency.</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Made tests and bug fixes of AI agents web analytics. Got new feedback from Quality Control Head. Made them tasks and did them.</t>
+          <t>Ran tests and fixed bugs in the AI agents web analytics. Also received new feedback from the Head of Quality Control, turned it into tasks and completed them.</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Started creating the backend from 0 for AI agents' scores web, because every time getting the data from Google Sheets is a very heavy and not-optimal process.</t>
+          <t>Started creating the backend for the AI agents score website from scratch, because retrieving the data from Google Sheets every time is a very heavy and non-optimal process.</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Created Supabase database table, uploaded the data to that table, and started making an automatically updating n8n workflow, so the website will have fresh data.</t>
+          <t>Created a Supabase database table, uploaded the data to it, and started building an automatically updating n8n workflow, so that the website always has fresh data.</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Made a little research on offline Telegram overall usage and bots. Continued creating backend database using PostgreSQL for the AI agents scores website.</t>
+          <t>Carried out a small piece of research into offline Telegram usage and bots in general. Also continued creating the backend database with PostgreSQL for the AI agents score website.</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Deployed successfully. Backend database integrating on AI Agents Score website. Still needs some optimization and integrating the paid database.</t>
+          <t>Deployed successfully and integrated the backend database into the AI Agents Score website. It still needs some optimization and the integration of the paid database.</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Continued creating backend for 'AI Agents Score' website.</t>
+          <t>Continued creating the backend for the AI Agents Score website.</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Started creating a workflow to automate some actions of the QA using Python and Bash commands.</t>
+          <t>Started creating a workflow to automate some of the QA actions using Python and Bash commands.</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Created QA automation code which automated the flow of the manual QA engineers.</t>
+          <t>Created QA automation code that automates the manual QA engineers' flow.</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Researched and made some different cases of QA automation project. Also made one case using other auto browser and did some tasks regarding Quality Control department.</t>
+          <t>Researched and built several different cases for the QA automation project. Also built one case using another automated browser, and completed several tasks for the Quality Control department.</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Got tasks from Head of Quality Control. Started working on them. Also, I have done some tasks regarding the automation QA for finishing the first part of the user's registration phase.</t>
+          <t>Received tasks from the Head of Quality Control and started working on them. Also completed several tasks on the QA automation, finishing the first part of the user registration phase.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Updated AI Agents Scores Website. Optimized and improved weights as needed. Continuing QA automation task. User email verification and registration last phase.</t>
+          <t>Updated the AI Agents Score website and optimized and improved the weights as required. Also continued the QA automation task — user email verification and the final registration phase.</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Optimized and made faster AI Agents. Scored websites' data loadings. Made a lot of steps further regarding QA Automation. It now creates a user, verifies email, inputs user bio data, only left passport confirmation.</t>
+          <t>Optimized and speeded up the data loading of the AI Agents Score website. Also made significant progress on the QA automation: it now creates a user, verifies the email and enters the user's bio data — only passport confirmation is left.</t>
         </is>
       </c>
     </row>
@@ -1408,8 +1408,8 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Made some attempts to improve Automation QA workflow.
-Added a new "good" positive feedback (with the correct n8n webhook URL call) feature to the AI Agents Score website.</t>
+          <t>Made several attempts to improve the QA automation workflow.
+Also added a new "good" positive feedback feature (with the correct n8n webhook URL call) to the AI Agents Score website.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Finished the QA automation's first project, and deployed to the QA Team lead's computer. It works perfectly. Caught errors, fixed them, and made the code maximally robust.</t>
+          <t>Finished the first QA automation project and deployed it on the QA team lead's computer, where it works perfectly. Also caught and fixed errors and made the code as robust as possible.</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Cleared code of the automation QA, also made the flow more clear.</t>
+          <t>Cleaned up the QA automation code and made the flow clearer.</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Updated the QA flow. Now it handles more flexibility in failing cases and avoids fails with reloading. Moving on to the next phases.</t>
+          <t>Updated the QA flow. It now handles failing cases more flexibly and avoids failures by reloading. Moving on to the next phases.</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>got new tasks to automate the QA for the next week ,and started doing it by adding some new steps in the automation flow, alsow made a alot of error catching and handling features.</t>
+          <t>Received new tasks to automate the QA for next week and started working on them by adding new steps to the automation flow. Also added a large number of error catching and handling features.</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>I have added a lot of things to the flow. Only the created parcel validation is left to finish the automation QA flow. Working on it, the other previously done steps and improvements were fixed, committed, validated, and made robust for errors.</t>
+          <t>Added a lot to the flow; only the created parcel validation is left in order to finish the QA automation flow, and work on it is in progress. The previously completed steps and improvements were fixed, committed, validated and made robust against errors.</t>
         </is>
       </c>
     </row>
@@ -1481,7 +1481,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Updated the automation QA flow. Made it more robust for the experience and overall bad cases. Still got one problem to fix.</t>
+          <t>Updated the QA automation flow and made it more robust for the user experience and for bad cases in general. One problem still remains to be fixed.</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1493,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Deployed backend for the AI-agents-score with Supabase. Working on optimizing it.</t>
+          <t>Deployed the backend for the AI Agents Score project with Supabase, and currently working on optimizing it.</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Made a new data table in Supabase. Made the data handling and corresponding data preprocessing automatic workflow which will parse and add the new data to the PostgreSQL of Supabase. Works perfectly. Continuing deployment of the backend for the AI-Agents-Score AI-powered website (that I have created from scratch).</t>
+          <t>Created a new data table in Supabase, and built the automatic workflow for data handling and the corresponding data pre-processing, which parses new data and adds it to the Supabase PostgreSQL database. It works perfectly. Also continued deploying the backend for the AI Agents Score AI-powered website that I created from scratch.</t>
         </is>
       </c>
     </row>
@@ -1517,8 +1517,8 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Successfully deployed Supabase backend for the AI-agents-scores website. Now the loading is way faster. Deleted unnecessary files, functions, graphs, variables, and other things regarding unnecessary graphs.
-Attended a meeting and got new tasks about Onex Georgia.</t>
+          <t>Successfully deployed the Supabase backend for the AI Agents Score website, so loading is now much faster. Also deleted unnecessary files, functions, graphs and variables related to the redundant graphs.
+Attended a meeting and received new tasks concerning ONEX Georgia.</t>
         </is>
       </c>
     </row>
@@ -1530,8 +1530,8 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Caught some errors, made bug fixes on AI-agents-score, did some tests of fixed bugs, then deployed the changes.
-Got new tasks about Onex Georgia region and city inputting problem, started working on it.</t>
+          <t>Caught several errors and fixed bugs on the AI Agents Score website, tested the fixes and deployed the changes.
+Also received new tasks about the region and city input problem for the ONEX Georgia region, and started working on them.</t>
         </is>
       </c>
     </row>
@@ -1543,9 +1543,9 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Finished Automation QA flow with all the cases, error handling, and robust automated flow. Deployed that on the QA Engineer's Computer.
-Got new tasks about other automated QA flow creating. 
-Started working on Projects Presentation Report.</t>
+          <t>Finished the QA automation flow with all of its cases, error handling and robust automated flow, and deployed it on the QA engineer's computer.
+Received new tasks about creating another automated QA flow.
+Started working on the projects presentation report.</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Updated The overall projects report-presentation and finished, also got new tasks regarding to Automation QA.</t>
+          <t>Updated and finished the overall projects report and presentation, and received new tasks regarding the QA automation.</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1569,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Went to 'Merdzavan' Warehouse and attended a meeting with the CEO of that warehouse. Understood their work with Excel files. Also, they showed me their work, so I will automate all the possible things for them. Also got new tasks about that automation and some materials that are to be sent to me.</t>
+          <t>Visited the Merdzavan warehouse and attended a meeting with its CEO. Learned how they work with Excel files, and they demonstrated their work so that I can automate everything possible for them. Also received new tasks about that automation, along with materials that are to be sent to me.</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Got tasks for Merdzavan automation, documented the task, created roadmap with deadline and started working on it. For all that, got new necessary materials to work with.</t>
+          <t>Received the tasks for the Merdzavan automation, documented them, created a roadmap with deadlines and started working on it. Also received the new materials needed for the work.</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Started creating n8n AI workflow for Merdzavan task. Also researching different ways to implement the task.</t>
+          <t>Started creating the n8n AI workflow for the Merdzavan task, and researched different ways of implementing it.</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Continued crafting AI n8n workflow for 'Merdzavan', also made manual data preprocessing for AI agents system prompt, which will be used in the same AI agent workflow.</t>
+          <t>Continued crafting the AI n8n workflow for Merdzavan, and also performed manual data pre-processing for the AI agent's system prompt, which will be used in the same AI agent workflow.</t>
         </is>
       </c>
     </row>
@@ -1617,7 +1617,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Finished creating the main working phase of the n8n agentic AI workflow. Waiting for approval to continue working on Telegram bot implementation.</t>
+          <t>Finished creating the main working phase of the n8n agentic AI workflow. Waiting for approval in order to continue with the Telegram bot implementation.</t>
         </is>
       </c>
     </row>
@@ -1629,8 +1629,8 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Almost done the AI n8n workflow for the Merdzavan automation, only left some tests on real data and deploying to work with the Telegram bot.
-Also got some tasks for further QA automation and a further meeting with team leads and CITO/CTO about AI integrating for the whole IT department (QA, Back-team, Front-team).</t>
+          <t>Almost finished the AI n8n workflow for the Merdzavan automation; only some tests on real data and deployment with the Telegram bot are left.
+Also received several tasks for further QA automation, and arranged a further meeting with the team leads and the CITO/CTO about integrating AI across the whole IT department (QA, backend team and frontend team).</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Created Telegram bot and connected to the n8n. Now it is getting the file and processing it batch by batch and outputting the necessary corresponding answer to the user. The 'Memory' of the AI agent needs to be improved and the bot will be ready.</t>
+          <t>Created a Telegram bot and connected it to n8n. It now receives the file, processes it batch by batch and returns the corresponding answer to the user. The AI agent's memory needs to be improved, after which the bot will be ready.</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Upgraded and improved the overall logic of the Telegram bot's AI n8n agentic workflow. Now it handles the file better.</t>
+          <t>Upgraded and improved the overall logic of the Telegram bot's AI n8n agentic workflow. It now handles the file better.</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Created three web version games for the Smart Wall screens, so the users can play the game and not be bored of the waiting for their package.</t>
+          <t>Created three web-based games for the Smart Wall screens, so that users can play while waiting for their package instead of being bored.</t>
         </is>
       </c>
     </row>
@@ -1678,7 +1678,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Made more games for Smart Wall (web versions), updated, fixed errors of the Merdzavan Telegram bot and Onex-AI-AGETS self-improving agents.</t>
+          <t>Created more games for the Smart Wall (web versions), and updated and fixed errors in the Merdzavan Telegram bot and the ONEX AI Agents self-improving agents.</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Improved the 'Catch the Parcels' smart wall game, made it full screen, and removed all user touch elements. Updated and improved the AI-Agents-Score website corresponding to the feedback got from QC agents. Updated and corrected the addresses of the corresponding communities of the agentic AI Telegram bot for the Merdzavan.</t>
+          <t>Improved the "Catch the Parcels" Smart Wall game, made it full screen and removed all user touch elements. Updated and improved the AI Agents Score website according to the feedback received from the QC agents. Also updated and corrected the addresses of the corresponding communities in the agentic AI Telegram bot for Merdzavan.</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Created new game "ONEX_parcel_way", updated all the other games to be fullscreened and improved. Bug fixed. Also updated the Merdzavan Telegram AI agentic bot's AI agent's memory (corrected addresses, made JSON with the necessary structure parsed from the CSV).</t>
+          <t>Created a new game, "ONEX Parcel Way", and updated all of the other games to be full screen and improved. Also fixed bugs and updated the memory of the Merdzavan Telegram AI agentic bot's AI agent (corrected the addresses and created JSON with the necessary structure, parsed from the CSV).</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Made all the smart wall games to get the username, tracking number, order number, etc. Deployed the fully working and updating AI agent's prompt improver AI workflow (made a backup copy of the AI agent prompt in DB (which is n8n data table), in case of prompt being spoiled).</t>
+          <t>Made all of the Smart Wall games capture the username, tracking number, order number, and so on. Also deployed the fully working AI agent prompt improver AI workflow, which updates the prompt and creates a backup copy of the AI agent's prompt in the database (an n8n data table), in case the prompt is spoiled.</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Upgraded the smart wall games. Now it mocks the user QR scanning and starts the game (QR scan triggers the game to start). The user chooses the game and starts playing. Got the necessary materials to trigger the game to end and started working on it.</t>
+          <t>Upgraded the Smart Wall games. They now mock the user's QR scanning and start the game (the QR scan triggers the game to start): the user chooses a game and starts playing. Also received the materials needed to trigger the end of the game and started working on it.</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Updated Merdzavan Telegram AI bot's agent's memory about correct addresses and deployed, waiting for the feedback.</t>
+          <t>Updated the Merdzavan Telegram AI bot agent's memory with the correct addresses and deployed it; waiting for feedback.</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Updated the Telegram bot AI agent's prompts memory (corrected addresses). Started data cleaning.</t>
+          <t>Updated the Telegram bot AI agent's prompt memory (corrected the addresses), and started data cleaning.</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Updated the Smart Wall games. Now they are getting "Your order is ready" trigger and ending the game. Also updated and corrected the addresses of the Merdzavan Telegram AI agentic bot's n8n workflow's AI agent's memory.</t>
+          <t>Updated the Smart Wall games. They now receive the "Your order is ready" trigger and end the game. Also updated and corrected the addresses in the AI agent's memory in the Merdzavan Telegram AI agentic bot's n8n workflow.</t>
         </is>
       </c>
     </row>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Met with the head of Quality Control to get the new requirements. Added a per-agent LEVEL 1 Avg Score on Agent Details, made every criterion clickable for Edit Score (persisted to Supabase) and Give Feedback (sends &lt;criterion description&gt; - &lt;feedback&gt; to n8n), and wired default cluster weights to be fetched live from the webhook.</t>
+          <t>Met with the Head of Quality Control in order to receive the new requirements. Added a per-agent LEVEL 1 average score in Agent Details, made every criterion clickable for Edit Score (persisted to Supabase) and Give Feedback (which sends &lt;criterion description&gt; - &lt;feedback&gt; to n8n), and wired the default cluster weights to be fetched live from the webhook.</t>
         </is>
       </c>
     </row>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Updated Merdzavan Telegram bot's addresses (AI agent's memory) and deployed. Updated and validated, then deployed AI-Agents-Scores' all the AI agents' prompts, and some UI and technical things.</t>
+          <t>Updated the Merdzavan Telegram bot's addresses (the AI agent's memory) and deployed them. Also updated, validated and deployed all of the AI Agents Score agents' prompts, together with some UI and technical changes.</t>
         </is>
       </c>
     </row>
@@ -1798,8 +1798,8 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Scraped and collected the necessary information about ONEX support agents and informations that she/he should know. Cleaned and made them in a nice state to give to AI in the future. 
-Also updated the n8n AI workflow and am now handling the 'connection lost' or 'closed the chat messages' cases with AI agents, and the prompts are working correctly.</t>
+          <t>Scraped and collected the necessary information about the ONEX support agents and the information that they should know. Cleaned it and brought it into a good state, ready to be given to the AI in the future.
+Also updated the n8n AI workflow, which now handles the "connection lost" and "customer closed the chat" cases with the AI agents, and the prompts work correctly.</t>
         </is>
       </c>
     </row>
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Cleaned, concatenated, and added the necessary information to the analyst AI agent of the AI-agents-scores about the Onex privacy and policy, and all the right and correct procedures about making some orders (and not only) using Onex.</t>
+          <t>Cleaned, concatenated and added the necessary information to the analyst AI agent of the AI Agents Score project regarding the ONEX privacy policy and the correct procedures for placing orders (and more) with ONEX.</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Researched ways of making happen to 'Checking 10 new tickets' after giving feedback to the AIAgent. Now it is in the testing phase. Not deployed yet.</t>
+          <t>Researched ways of implementing the "check 10 new tickets" step after feedback is given to the AI agent. It is now in the testing phase and has not been deployed yet.</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Updated the database of the AI agents' scores and made a lot of UI updates. Deployed the new feature of seeing the 10 thickest after the feedback given. Made the UI user-friendly and easy to understand.</t>
+          <t>Updated the AI agents score database and made a large number of UI updates. Deployed the new feature that shows the next 10 tickets after feedback is given, and made the UI user-friendly and easy to understand.</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Updated some addresses of the Merdzavan bot automation and deployed the new memory with the updated correct addresses of the Telegram bot.</t>
+          <t>Updated some of the Merdzavan bot automation addresses, and deployed the Telegram bot's new memory with the corrected addresses.</t>
         </is>
       </c>
     </row>
@@ -1859,9 +1859,9 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Updated the "Send Another Feedback" window to display the associated feedback criteria for each submitted feedback entry (e.g., Feedback #1 – Criteria Name, Feedback #2 – Criteria Name).
-Added a "View Thicket Grades" button in the Next 10 Thickets section of Thicket Feedback.
-Enhanced Edit Criteria Score by adding an "N/A" option to prevent zero scores from negatively affecting the average score calculation.</t>
+          <t>Updated the "Send Another Feedback" window so that it displays the associated feedback criteria for each submitted feedback entry (for example, Feedback #1 – criterion name, Feedback #2 – criterion name).
+Added a "View Ticket Grades" button in the Next 10 Tickets section of Ticket Feedback.
+Enhanced Edit Criteria Score by adding an "N/A" option, in order to prevent zero scores from negatively affecting the average score calculation.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Adding new functionality to the AI-Agents-Scores website, so when a user makes feedback, it will change that exact thicket with new updated and validated grades and analysis, and highlight the thicket, so the user should know that the thicket was given feedback.</t>
+          <t>Added new functionality to the AI Agents Score website, so that when a user submits feedback, that exact ticket is updated with new validated grades and analysis, and the ticket is highlighted so that the user knows feedback has been given for it.</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Updated the UI of the search bar of the AI-Agents-Scores website's 'Tickets' section. Updated the structure of the tickets in the backend of the website (PostgreSQL Supabase data table), added new columns, and made them change UI so the user can separate the tickets that have been feedbacked and the tickets that have not. All the changes were deployed.</t>
+          <t>Updated the UI of the search bar in the "Tickets" section of the AI Agents Score website. Also updated the structure of the tickets in the website's backend (the Supabase PostgreSQL data table), added new columns and reflected them in the UI, so that users can distinguish the tickets that have received feedback from those that have not. All changes were deployed.</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Starting making of 3 AI agents (actually 4) out of one AI agent, so the work will be done in higher quality and simpler, with faster and shorter prompts. Still working on it, testing, not deployed.</t>
+          <t>Started splitting one AI agent into three (in fact four) AI agents, so that the work is done at higher quality and more simply, with faster and shorter prompts. Still in progress and being tested; not deployed yet.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Continuing creating AI robust agents, separating the levels as one AI agent each so there will be less prompt, light work and high quality. Still not finished, not deployed.</t>
+          <t>Continued creating robust AI agents, separating the levels so that each level has its own AI agent, which means shorter prompts, lighter work and higher quality. Not finished and not deployed yet.</t>
         </is>
       </c>
     </row>
@@ -1921,8 +1921,8 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Continued working on new separated level analyzer agents, made a lot of updates and improvements and deployed. 
-Started working on ONEX users level updating/adding also.</t>
+          <t>Continued working on the new separated level analyzer agents, made a large number of updates and improvements, and deployed them.
+Also started working on updating and adding ONEX user levels.</t>
         </is>
       </c>
     </row>
@@ -1934,8 +1934,8 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>updated self improving ai agentic n8n workflow made some testes, level 1 analyst updating is done, level 2 and 3 left. 
-also made some researches and tests for searching and updating ONEX user levels(the new update).</t>
+          <t>Updated the self-improving AI agentic n8n workflow and ran several tests; the level 1 analyst update is done, and levels 2 and 3 are left.
+Also carried out research and tests on searching for and updating ONEX user levels (the new update).</t>
         </is>
       </c>
     </row>
@@ -1947,7 +1947,7 @@
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>updated and almost finished self improving AI agentic workflow of the ai-agents-score, needs some tests and deploy.</t>
+          <t>Updated and almost finished the self-improving AI agentic workflow of the AI Agents Score project; it still needs some tests and deployment.</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>Made update on self improving ai agentic workflow, tested, validated and made them robust, deployed, and ready to real-life tests.</t>
+          <t>Updated the self-improving AI agentic workflow, tested and validated it, made it robust and deployed it, and it is now ready for real-life tests.</t>
         </is>
       </c>
     </row>
@@ -1971,8 +1971,8 @@
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>added, tested, validated and deployed the last ui and backend+logic updates of the new self-improving AI workflow.
-started working on clusterizing tickets by their topics as a continuation of the self-improving agents and tracking their quality.</t>
+          <t>Added, tested, validated and deployed the latest UI, backend and logic updates of the new self-improving AI workflow.
+Also started working on clustering tickets by topic, as a continuation of the self-improving agents and the tracking of their quality.</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>Added a per-ticket topic to the 'ai-agents-scores' system — surfaced as a dedicated column and detail box on the Tickets page — by plumbing a new topic database column through the tickets-snapshot edge function and ticket parser. Reworked the post-feedback "Feedback Watch" to cluster by topic instead of agent, so after any correction it tracks the next 10 same-topic tickets graded afterwards, letting us verify whether the AI learned and applied the correction to similar tickets.</t>
+          <t>Added a per-ticket topic to the AI Agents Score system — shown as a dedicated column and detail box on the Tickets page — by plumbing a new topic database column through the tickets snapshot edge function and the ticket parser. Also reworked the post-feedback "Feedback Watch" so that it clusters by topic instead of by agent: after any correction it tracks the next 10 tickets on the same topic that are graded afterwards, which makes it possible to verify whether the AI learned the correction and applied it to similar tickets.</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>Corrected the topic setter ai agent’s prompt, added one topic and deployed that.</t>
+          <t>Corrected the topic setter AI agent's prompt, added one topic and deployed the change.</t>
         </is>
       </c>
     </row>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>did testes and some tracks for the new ai agentic n8n workflow of analyzing and grading tickets(customer support workers).</t>
+          <t>Ran tests and traced the new AI agentic n8n workflow for analyzing and grading tickets (customer support workers).</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>making qa-automation from dev/staging to live. Fixed the live-verification bug and the WSL venv setup failure, and made the WSL/Windows toolchains coexist cleanly.</t>
+          <t>Moved the QA automation from dev/staging to live. Fixed the live verification bug and the WSL virtual environment setup failure, and made the WSL and Windows toolchains coexist cleanly.</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>did meeting with QA team's teamlead and got new tasks, also showcased the new automation flow got positive feedback. Starting working on the new qa's flow(not new but additional).</t>
+          <t>Held a meeting with the QA team's team lead and received new tasks. Also showcased the new automation flow and received positive feedback, and started working on the QA's new (additional) flow.</t>
         </is>
       </c>
     </row>
@@ -2044,8 +2044,8 @@
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>I have officially started development on the ONEX Academy project. The goal is to build an engaging, quiz-based web app for support agents to test their knowledge. 
-Also i continue working updating testing and deploying the qa-automation project for the user and parcel creation box creating and addition etc... we have some cases that needs to be reviewed and corrected.</t>
+          <t>Officially started development of the ONEX Academy project. The goal is to build an engaging, quiz-based web app that support agents can use to test their knowledge.
+Also continued updating, testing and deploying the QA automation project for user and parcel creation, box creation and addition, and so on; some cases still need to be reviewed and corrected.</t>
         </is>
       </c>
     </row>
@@ -2057,8 +2057,8 @@
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>updated live qa-automation flow, deployed in the qa team lead's pc, tested it.
-made meeting with quality control team and got tasks, showed the project prototype of that.</t>
+          <t>Updated the live QA automation flow, deployed it on the QA team lead's PC and tested it.
+Also held a meeting with the quality control team, received tasks and showed them the prototype of the project.</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>created, tested, and deployed task scheduler to send all the new images to amazon AWS S3 server and store them with working urls.</t>
+          <t>Created, tested and deployed a task scheduler that sends all new images to the Amazon AWS S3 server and stores them with working URLs.</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Built 11 new academy features (media questions, timers, topics, multi-correct, levels, link/roadmap, explanations, timing analytics, screenshot deterrence) and removed flashcards. After accidentally applying the schema to the live "Agents Tickets" DB (since restored), we set up a dedicated Supabase project (imzedtezqkqrynjzvcxq) and pointed the app at it. Left to do: publish in Lovable and add the onex@onex.am admin.</t>
+          <t>Built 11 new academy features (media questions, timers, topics, multi-correct answers, levels, link/roadmap, explanations, timing analytics and screenshot deterrence) and removed the flashcards. After the schema was accidentally applied to the live "Agents Tickets" database (since restored), set up a dedicated Supabase project (imzedtezqkqrynjzvcxq) and pointed the app at it. Left to do: publish in Lovable and add the onex@onex.am admin.</t>
         </is>
       </c>
     </row>
@@ -2094,8 +2094,8 @@
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>I synced the DB schema, types, and RPCs, and fixed scoring, auth, and gameplay bugs. You ran the SQL; now just create the quiz-media storage bucket.
-Also made some tests and updated, improved, fixed bugs, made improvements, and deployed.</t>
+          <t>Synced the database schema, types and RPCs, and fixed scoring, authentication and gameplay bugs. The SQL has been run; the only remaining step is to create the quiz media storage bucket.
+Also ran tests, made updates and improvements, fixed bugs and deployed.</t>
         </is>
       </c>
     </row>
@@ -2107,8 +2107,8 @@
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>got some feedback about onex-academy.
-tested and got new task for amazon s3 bucket import automation for images to have urls.</t>
+          <t>Received feedback on ONEX Academy.
+Also ran tests and received a new task for the Amazon S3 bucket import automation, so that the images have URLs.</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2120,7 @@
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>made tests and improvements and deployed the amazon bucket automatic image uploader.</t>
+          <t>Ran tests and improvements and deployed the automatic image uploader for the Amazon S3 bucket.</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>made tests and improvements and deployed the amazon bucket automatic image uploader.</t>
+          <t>Ran tests and improvements and deployed the automatic image uploader for the Amazon S3 bucket.</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Built a Google Sheets weekly timesheet with 5-minute time dropdowns (07:00 onward) for Start/End times that automatically calculate and sum each person's worked hours in the SUMMARY column.</t>
+          <t>Built a weekly timesheet in Google Sheets with five-minute time dropdowns (from 07:00 onwards) for the start and end times, which automatically calculate and sum each person's worked hours in the SUMMARY column.</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>fixed the google sheets dropdown button time setting issue, made it robust and flexible</t>
+          <t>Fixed the time setting issue with the Google Sheets dropdown button, and made it robust and flexible.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>created and deployed amazon s3 bucket import automation for images to have urls on the other pc, just need to set amazon cridentials using terminal and one pc left to do the same task</t>
+          <t>Created and deployed the Amazon S3 bucket import automation on another PC, so that the images have URLs; the only remaining steps are to set the Amazon credentials via the terminal and to perform the same task on one more PC.</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
         <is>
           <t>Added AI free-text grading using the Gemini 3 Flash model.
 Enabled custom question points and resolved the image upload issue.
-Added one task scheduled to the other pc of onex china for amazon upload automating task.</t>
+Also added a scheduled task on another ONEX China PC for the Amazon upload automation task.</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Fixed free-text quiz questions not showing an answer input field. Consolidated to one Supabase project and applied the database migration. Fixed dev environment loading, enabling AI grading to work correctly.</t>
+          <t>Fixed the issue where free-text quiz questions did not show an answer input field. Consolidated everything into a single Supabase project and applied the database migration. Also fixed the loading of the dev environment, which enabled AI grading to work correctly.</t>
         </is>
       </c>
     </row>
@@ -2206,8 +2206,8 @@
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>updated the last computer of the onex-china, so now all the parcels with tracking code in china should be automatically uploaded to the amazon s3 bucket database and get url's with them.
-made meeting with chief quality control head and got new tasks and feedback about the AI-powered onex-academy quiz website. and did some major updates to that, tested and deployed.</t>
+          <t>Updated the last ONEX China computer, so all parcels with a tracking code in China are now automatically uploaded to the Amazon S3 bucket database and receive URLs.
+Also held a meeting with the chief head of quality control, received new tasks and feedback about the AI-powered ONEX Academy quiz website, and made major updates to it, tested them and deployed.</t>
         </is>
       </c>
     </row>
@@ -2219,9 +2219,9 @@
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>added two new features to the onex-academy project.
-1. added skpi feature so the user can skip and see the question's right answer
-2. added new section so the admin can grade and set score manually the questions that the AI failed to grade.</t>
+          <t>Added two new features to the ONEX Academy project:
+1. Added a skip feature, so that users can skip a question and see its correct answer.
+2. Added a new section, so that admins can manually grade and set the score for the questions that the AI failed to grade.</t>
         </is>
       </c>
     </row>
@@ -2233,11 +2233,11 @@
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>worked on adding ONEX.am watermark on the images of the amazon s3 bucket autouploading. needs further tests updated and deployment.
-added 4 new features to the onex-academy project:
-1. memory match starts with a few seconds open-fliped so the users can remember the sides of cards
-2. memory quiz cards' numbers are now adjustable and customable set for the admin(admin decides the number of the memory cards)
-3. when adding new quiz or sth else, the tab closing opening or reoading or switching the other tab doesn't vanish the entered/inputted text, uploaded file, etc.</t>
+          <t>Worked on adding the ONEX.am watermark to the images in the Amazon S3 bucket auto-uploading process; it still needs further tests, updates and deployment.
+Also added four new features to the ONEX Academy project:
+1. The memory match game now starts with the cards flipped open for a few seconds, so that users can memorize their positions.
+2. The number of memory quiz cards is now adjustable and customizable by the admin (the admin decides how many memory cards there are).
+3. When adding a new quiz or anything else, closing, opening or reloading the tab, or switching to another tab, no longer clears the entered text, uploaded files, and so on.</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>tested and validated the onex-academy website to be safe that is deployed.</t>
+          <t>Tested and validated the ONEX Academy website in order to make sure that it is safely deployed.</t>
         </is>
       </c>
     </row>
@@ -2261,7 +2261,7 @@
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>started working on deploying the project of amazon s3 bucket uploading automation, which includes quality decreasing and watermark adding(needs to download python on the onex-china computers so the code should work)</t>
+          <t>Started deploying the Amazon S3 bucket upload automation project, which includes image quality reduction and watermark adding (Python needs to be installed on the ONEX China computers in order for the code to work).</t>
         </is>
       </c>
     </row>
@@ -2273,8 +2273,8 @@
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>continue working on s3 amazon bucket autouploading on onex-china computers,
-also starter working on footdraw.com's article maker n8n AI agentic workflow.`</t>
+          <t>Continued working on the Amazon S3 bucket auto-uploading on the ONEX China computers.
+Also started working on the article maker n8n AI agentic workflow for footdraw.com.</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Successfully built an automated n8n workflow for FootDraw articles. It generates structured markdown content, SEO metadata, and custom images.</t>
+          <t>Successfully built an automated n8n workflow for FootDraw articles. It generates structured Markdown content, SEO metadata and custom images.</t>
         </is>
       </c>
     </row>
@@ -2298,8 +2298,8 @@
       </c>
       <c r="B150" s="3" t="inlineStr">
         <is>
-          <t>had meeting about general AI to use in ONEX.am overall team. 
-Tested, validated, improved and finished article make ai n8n  agentic workflow, started the AI translation agentic workflows' creating.</t>
+          <t>Held a meeting about the general use of AI across the ONEX.am team.
+Also tested, validated, improved and finished the AI article maker n8n agentic workflow, and started creating the AI translation agentic workflows.</t>
         </is>
       </c>
     </row>
@@ -2311,11 +2311,9 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>Built an n8n workflow to translate JSON using Gemini.
-The code parsed AI outputs, restored images, and mapped languages.
-did a tasks review and got new tasks and feedback for onex-academy wbsite.
-Built four ONEX-Academy features: wrong-answer Next button, auto-growing editor fields.
-Added AI quiz-summary debrief and email/Telegram new-user signup verification.</t>
+          <t>Built an n8n workflow that translates JSON using Gemini; the code parses the AI outputs, restores the images and maps the languages.
+Also carried out a task review and received new tasks and feedback for the ONEX Academy website.
+Built four ONEX Academy features: a Next button for wrong answers, auto-growing editor fields, an AI quiz summary debrief, and email and Telegram verification for new user signups.</t>
         </is>
       </c>
     </row>
@@ -2327,8 +2325,8 @@
       </c>
       <c r="B152" s="3" t="inlineStr">
         <is>
-          <t>updated the onex-academy websites card game number setting input field, made dynamically enlarging feature for text input fields, added website's ui text editing field.
-finished article translator workflow's ai agents prompts, code nodes, output parsers, all workflow is now tested, validated and deployed, now its translating in 7 different languages correctly and sends the webhook respons back correctly.</t>
+          <t>Updated the card game number setting input field on the ONEX Academy website, added a dynamic enlarging feature for text input fields, and added a UI text editing field to the website.
+Also finished the article translator workflow's AI agent prompts, code nodes and output parsers; the whole workflow has now been tested, validated and deployed, and it translates correctly into 7 different languages and returns the webhook response correctly.</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2338,7 @@
       </c>
       <c r="B153" s="3" t="inlineStr">
         <is>
-          <t>madedid meeting with the ctw, clarificated and managed tasks presenting and continued tasks for te day</t>
+          <t>Held a meeting with the CTO, clarified and organized the tasks, presented them, and continued with the tasks for the day.</t>
         </is>
       </c>
     </row>
@@ -2352,8 +2350,7 @@
       </c>
       <c r="B154" s="3" t="inlineStr">
         <is>
-          <t>AI test summary was silently failing with no diagnosable cause.
-Fixed error logging, clip-tolerant validation, and reliable model config.</t>
+          <t>Fixed the AI test summary, which was silently failing with no diagnosable cause, by correcting the error logging, adding clip-tolerant validation and making the model configuration reliable.</t>
         </is>
       </c>
     </row>
@@ -2365,8 +2362,8 @@
       </c>
       <c r="B155" s="3" t="inlineStr">
         <is>
-          <t>Enabled Telegram-based registration for ONEX Academy on its Lovable deployment. 
-Configured bot, migration, and webhook, then fixed and verified signup.</t>
+          <t>Enabled Telegram-based registration for ONEX Academy on its Lovable deployment.
+Configured the bot, the migration and the webhook, then fixed and verified the signup.</t>
         </is>
       </c>
     </row>
@@ -2378,9 +2375,9 @@
       </c>
       <c r="B156" s="3" t="inlineStr">
         <is>
-          <t>added new feature in the onex-academy:
-1. new badges with their icons/pictures
-2. new animation when level up and badges getting</t>
+          <t>Added new features to ONEX Academy:
+1. New badges with their own icons and pictures.
+2. New animations for levelling up and earning badges.</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2390,7 @@
       <c r="B157" s="3" t="inlineStr">
         <is>
           <t>Tested, validated and deployed the new badges and level animation feature.
-Added new ui updates on the onex-academy website project.</t>
+Also added new UI updates to the ONEX Academy website project.</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2402,7 @@
       </c>
       <c r="B158" s="3" t="inlineStr">
         <is>
-          <t>started owrking on onex-academy project website's mobile version</t>
+          <t>Started working on the mobile version of the ONEX Academy project website.</t>
         </is>
       </c>
     </row>
@@ -2417,7 +2414,7 @@
       </c>
       <c r="B159" s="3" t="inlineStr">
         <is>
-          <t>Added a dedicated mobile version mode without changing the desktop layout. Built a three-dots hamburger menu grouping play, leaderboard, and settings. Added a mobile text-size adjuster to enlarge quizzes and inputs. Improved the memory card game with red wrong-pair animation and click-flip fixes.</t>
+          <t>Added a dedicated mobile version mode without changing the desktop layout. Built a three-dots hamburger menu grouping play, leaderboard and settings. Added a mobile text size adjuster to enlarge quizzes and inputs. Improved the memory card game with a red wrong-pair animation and click-flip fixes.</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2426,7 @@
       </c>
       <c r="B160" s="3" t="inlineStr">
         <is>
-          <t>Updating and improving the website’s features, making it nicer, and more user friendly, working on testing and finding bugs, correcting and fixing them, then deploying, also working on the websites mobile versions improvements.</t>
+          <t>Updated and improved the website's features, making it nicer and more user-friendly, worked on testing and finding bugs, corrected and fixed them and deployed the changes, and also worked on improvements to the website's mobile version.</t>
         </is>
       </c>
     </row>
@@ -2441,8 +2438,8 @@
       </c>
       <c r="B161" s="3" t="inlineStr">
         <is>
-          <t>Built a new "Questions Database" quiz type serving random question subsets with per-week play limits. Added admin controls for pool size, limits, topic balancing, and per-player resets.
-Added an admin button to copy quiz questions into any Questions Database. Merged Lovable's security fixes with the feature and pushed to main.</t>
+          <t>Built a new "Questions Database" quiz type that serves random question subsets with per-week play limits. Added admin controls for the pool size, limits, topic balancing and per-player resets.
+Also added an admin button that copies quiz questions into any Questions Database, and merged Lovable's security fixes with the feature and pushed them to main.</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2451,7 @@
       </c>
       <c r="B162" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project.</t>
+          <t>Researched Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2463,7 @@
       </c>
       <c r="B163" s="3" t="inlineStr">
         <is>
-          <t>Continue Researcing for armenian stt models to use it in the ai-agents-scores quality control project.</t>
+          <t>Continued researching Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2475,7 @@
       </c>
       <c r="B164" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project - continue.</t>
+          <t>Continued researching Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2490,8 +2487,8 @@
       </c>
       <c r="B165" s="3" t="inlineStr">
         <is>
-          <t>Investigated, found the problem, fixed, updated and deployed the aI agentic “footdraw.com”’s translator n8n workflow, now it no loder makes 500 error.
-Updated aI agentic “footdraw.com”’s article maker n8n workflow, now it generates an image without an english(or any other language) text on the image.</t>
+          <t>Investigated, located and fixed the problem in the AI agentic translator n8n workflow for footdraw.com, then updated and deployed it; it no longer returns a 500 error.
+Also updated the AI agentic article maker n8n workflow for footdraw.com, which now generates images without English (or any other language) text on them.</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2500,7 @@
       </c>
       <c r="B166" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project. - continue</t>
+          <t>Continued researching Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2515,8 +2512,8 @@
       </c>
       <c r="B167" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project.
-Found some models to test with, created nice ui for browsing mp3 onex calls and model, and testing it locally.</t>
+          <t>Researched Armenian speech-to-text models for use in the AI Agents Score quality control project.
+Found several models to test with, created a neat UI for browsing the ONEX call MP3 files and the models, and tested it locally.</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2525,7 @@
       </c>
       <c r="B168" s="3" t="inlineStr">
         <is>
-          <t>In onex-academy replaced Telegram deep-link signup with a hashed six-digit confirmation code. Added confirm-password field showing a live check or cross icon. Code shipped to main; remaining blocker is the unapplied live migration.</t>
+          <t>Replaced the Telegram deep-link signup in ONEX Academy with a hashed six-digit confirmation code. Added a confirm-password field that shows a live tick or cross icon. The code has been shipped to main; the remaining blocker is the unapplied live migration.</t>
         </is>
       </c>
     </row>
@@ -2540,9 +2537,9 @@
       </c>
       <c r="B169" s="3" t="inlineStr">
         <is>
-          <t>Replaced the dead bot, removed email verification, registered the webhook.
-Added weekly play limits for every quiz, greying out exhausted cards.
-Built twice-weekly reminder bot plus admin panel; migrations await your dashboard.</t>
+          <t>Replaced the dead bot, removed the email verification and registered the webhook.
+Added weekly play limits for every quiz, greying out the exhausted cards.
+Built a twice-weekly reminder bot plus an admin panel; the migrations are awaiting the dashboard.</t>
         </is>
       </c>
     </row>
@@ -2554,9 +2551,9 @@
       </c>
       <c r="B170" s="3" t="inlineStr">
         <is>
-          <t>Swapped in new @AcademyONEXbot and registered its verification webhook.
-Fixed six-digit signup codes, auth, database and media-bucket security gaps.
-Added Bot Messages admin tab: reminders or free text, selected players.</t>
+          <t>Swapped in the new @AcademyONEXbot and registered its verification webhook.
+Fixed the six-digit signup codes and the authentication, database and media bucket security gaps.
+Added a Bot Messages admin tab for sending reminders or free text to selected players.</t>
         </is>
       </c>
     </row>
@@ -2568,10 +2565,10 @@
       </c>
       <c r="B171" s="3" t="inlineStr">
         <is>
-          <t>Replaced the Telegram bot; verification and webhook now work.
+          <t>Replaced the Telegram bot; the verification and webhook now work.
 Added an admin panel for sending Telegram reminders.
-Extracted Anna's chat requests; all outstanding site tasks done.
-Made an analysis of the onex-academy project, cleaned updated and improved the codebase.</t>
+Extracted Anna's chat requests; all outstanding site tasks are done.
+Also analyzed the ONEX Academy project and cleaned, updated and improved the codebase.</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2580,7 @@
       </c>
       <c r="B172" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project. - continue</t>
+          <t>Continued researching Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2592,7 @@
       </c>
       <c r="B173" s="3" t="inlineStr">
         <is>
-          <t>started creating the ai onex blog maker workflow with its web-version, so in future we can deploy it in the main onex website</t>
+          <t>Started creating the AI ONEX blog maker workflow together with its web version, so that it can be deployed on the main ONEX website in the future.</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2604,7 @@
       </c>
       <c r="B174" s="3" t="inlineStr">
         <is>
-          <t>Continuing creating ONEX.am blog making AI workflow.</t>
+          <t>Continued creating the ONEX.am blog making AI workflow.</t>
         </is>
       </c>
     </row>
@@ -2619,9 +2616,12 @@
       </c>
       <c r="B175" s="3" t="inlineStr">
         <is>
-          <t>Confirmed Tilda has no write API; chose self-hosted rendering instead.
-Built image offloading, slug publishing, SSR public pages, and Tilda hub.
-Pipeline runs end-to-end; first blog failed QA on hallucinated SEO.</t>
+          <t>Confirmed that Tilda has no write API, and chose self-hosted rendering instead.
+Built image offloading, slug publishing, SSR public pages and the Tilda hub.
+The pipeline runs end to end; the first blog post failed QA because of hallucinated SEO.
+Updated the ONEX Academy website.
+Added a new feature for uploading more than one image and link.
+Added a new feature for viewing all of the AI agents' prompts on the website, which the admin can edit.</t>
         </is>
       </c>
     </row>
@@ -2633,9 +2633,9 @@
       </c>
       <c r="B176" s="3" t="inlineStr">
         <is>
-          <t>Confirmed Tilda has no write API; built three export routes instead.
-Shipped image offloading, publishing, SSR pages, hub block, HTML export.
-Rewrote nodes 10, 13, 17 around your proven Avengers page format.</t>
+          <t>Confirmed that Tilda has no write API, and built three export routes instead.
+Shipped image offloading, publishing, SSR pages, the hub block and HTML export.
+Rewrote nodes 10, 13 and 17 around the proven Avengers page format.</t>
         </is>
       </c>
     </row>
@@ -2647,7 +2647,7 @@
       </c>
       <c r="B177" s="3" t="inlineStr">
         <is>
-          <t>updated the onex ai blog autiamtmaker's automation and showed to the corresponding professional</t>
+          <t>Updated the automation of the ONEX AI blog auto-maker and demonstrated it to the corresponding specialist.</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
       </c>
       <c r="B178" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project.</t>
+          <t>Researched Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2671,7 @@
       </c>
       <c r="B179" s="3" t="inlineStr">
         <is>
-          <t>Researched for armenian stt models to use it in the ai-agents-scores quality control project.</t>
+          <t>Researched Armenian speech-to-text models for use in the AI Agents Score quality control project.</t>
         </is>
       </c>
     </row>
@@ -2683,9 +2683,7 @@
       </c>
       <c r="B180" s="3" t="inlineStr">
         <is>
-          <t>I met with quality control heads and got fifteen tasks. I will complete these
-necessary changes by early next week. Once ready, I will notify you for another
-testing session.</t>
+          <t>Met with the quality control heads and received fifteen tasks. These necessary changes will be completed by early next week, and once they are ready I will notify you for another testing session.</t>
         </is>
       </c>
     </row>
@@ -2698,31 +2696,31 @@
       <c r="B181" s="3" t="inlineStr">
         <is>
           <t>Badges
-Added badges admins can award by hand, with picture and text
-Users now see locked badges blurred, with progress shown
-Telegram sends a message for every new badge earned
+Added badges that admins can award by hand, with a picture and text.
+Users now see locked badges blurred, with their progress shown.
+Telegram sends a message for every new badge earned.
 Memory game
-Game continues to the next round until all pairs played
-Each round has its own timer, scores add up
-Fixed card layout on phones so it fits the screen
+The game now continues to the next round until all pairs have been played.
+Each round has its own timer, and the scores add up.
+Fixed the card layout on phones so that it fits the screen.
 Quizzes
-Free-text quizzes now ask "chat or call" before starting
-Chat mode warns about spelling, punctuation and emoji use
-Chat mode grading now checks spelling and punctuation too
-Popup shows the quiz time limit for five seconds
-Quiz descriptions show in full, no cut-off dots
-Every quiz can have its own uploaded icon picture
+Free-text quizzes now ask "chat or call" before starting.
+Chat mode warns about spelling, punctuation and emoji use.
+Chat mode grading now checks spelling and punctuation as well.
+A popup shows the quiz time limit for five seconds.
+Quiz descriptions are shown in full, with no cut-off ellipsis.
+Every quiz can have its own uploaded icon picture.
 Admin panel
-New "Users" page with full details for each person
-Admins can edit any question's score and correct/wrong mark
-Admins see who is online and playing right now
-Admins see each question's time spent and answer times
-Fixed table so names and scores are no longer cut off
+Added a new "Users" page with full details for each person.
+Admins can edit any question's score and its correct or wrong mark.
+Admins can see who is online and playing right now.
+Admins can see the time spent on each question and the answer times.
+Fixed the table so that names and scores are no longer cut off.
 Telegram bot
-Sends round score, total points and AI feedback after playing
-Removed all "/stop" mentions from bot messages
+Sends the round score, total points and AI feedback after playing.
+Removed all "/stop" mentions from the bot messages.
 Login
-Password fields got show/hide eye and copy buttons</t>
+Added show/hide eye and copy buttons to the password fields.</t>
         </is>
       </c>
     </row>
@@ -2735,124 +2733,206 @@
       <c r="B182" s="3" t="inlineStr">
         <is>
           <t>1. Answers with text, link and picture
-Admins can now pick, per question, how the player answers: free text, link, picture, or any mix. Each ticked box gets its own "correct answer" field, and the AI compares every part the player submits — including looking at their screenshot — into one score.
-Players see exactly the inputs the admin chose, can paste a screenshot with Ctrl+V, and their link/picture shows up in the review screen and in the admin grading queue.
+Admins can now choose, per question, how the player answers: free text, link, picture, or any combination. Each ticked box gets its own "correct answer" field, and the AI compares every part that the player submits — including looking at their screenshot — into a single score.
+Players see exactly the inputs that the admin chose, can paste a screenshot with Ctrl+V, and their link or picture appears in the review screen and in the admin grading queue.
 2. Bot messages can be sent again
-"Run now for everyone" was blocked after the first press (that's why it said "Sent 0 of 0"). Now it sends every time you press it. The automatic twice-weekly reminder still sends only once per person per day.
+"Run now for everyone" was blocked after the first press, which is why it said "Sent 0 of 0". It now sends every time the button is pressed. The automatic twice-weekly reminder still sends only once per person per day.
 3. Quiz time warning
-When any quiz starts, a ~5 second popup shows the time for the whole quiz. If the quiz has no overall limit, it adds up the question timers and shows that total instead. Timers were already settable by admins, so nothing new was needed there.
+When any quiz starts, a popup shows the time for the whole quiz for about five seconds. If the quiz has no overall limit, it adds up the question timers and shows that total instead. The timers were already settable by admins, so nothing new was needed there.
 4. Cleanup
-Deleted 33 old SQL files, a stale second lockfile, and leftover build folders — after checking that full_setup.sql still contains the complete database. Repo is 31% smaller (186 → 153 files). Also cut about a fifth of the code comments, keeping the ones that explain real gotchas.
-Enlarged dashboard quiz card images from 48px to 80-96px wide.
+Deleted 33 old SQL files, a stale second lockfile and leftover build folders, after checking that full_setup.sql still contains the complete database. The repository is 31% smaller (186 → 153 files). Also removed about a fifth of the code comments, keeping the ones that explain real gotchas.
+Enlarged the dashboard quiz card images from 48px to 80–96px wide.
 Added multi-picture uploads with corner remove buttons for admins and players.
 Added an admin "prompt for AI" checkbox on open-answer questions.
-[agents-ai-scores] made a new "finish and send" feedback button, so admin wont be waitinf after every single feedback, to process, tehn send again.</t>
+[AI Agents Score] Created a new "finish and send" feedback button, so that the admin does not have to wait for processing after every single piece of feedback before sending again.</t>
         </is>
       </c>
     </row>
     <row r="183" ht="57.6" customHeight="1">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>10/08/2026 15:21:00</t>
+          <t>21/08/2026 15:24:29</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
         <is>
-          <t>updated the onex-academy website
-added new feature to uploade more than one images and links
-new feature to see all the prompts of the ai agents in the website, admin can edit  them all</t>
+          <t>[ONEX Academy]
+Added a picture zoom feature to the questions, so that users can view them full screen, with a zoom button (including + and - buttons) to zoom in on a picture and read the text or handwritten content.
+Enabled pasting text into the question answer field with a right mouse click.
+Added a new feature for adding clickable links and icons (pictures) to question prompts — clickable text in two ways: a plain clickable link, and a text that is clickable and has a link underneath it, with the admin deciding which option to use when creating the question — so that users can click the link or the clickable picture in the question, go to the website and then answer the question.
+Fixed the link comparison issue.
+Fixed the model's picture blindness (the user attached a picture, but the AI agent did not see it).
+Changed the "Try again" button to "Proceed to the next question" when a wrong answer is clicked in multiple-choice questions.
+[AI Agents Score]
+Added a new "AI agents" section to the AI Agents Score website, so that the admin can see all of the AI agents' prompts and edit them as required (created two n8n workflows for this task, with two webhooks: POST to update the AI agents' prompts, and GET to read and display them on the website).</t>
         </is>
       </c>
     </row>
     <row r="184" ht="244.8" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>21/08/2026 15:24:29</t>
+          <t>24/08/2026 15:57:23</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
         <is>
-          <t>[onex-academy]
-Picture zoom feature in the questions for the users, so they can see them in full screen, and zoom button with maybe + and - buttons to zoom the picture and see the text or handwritten things, etc.
-Paste the text using mouse right click in question answer field
-Add a new feature which will be able to add Clickable links and icons(pictures) in question prompts (clickable text in two ways, just clickable link, and a text which is clickable and under that have a link, admin decides which way when creating question, so users can click that link in the question or the clickable picture, get in the website, then answer the question)
-fix the links comparison issue
-fix picture blindness of the model (user attached picture, but the ai agent did not see it)
-Change &lt;&lt;try again&gt;&gt; button to &lt;&lt;proceed to the next question&gt;&gt; when clicking wrong answer in the multiple questions type of question
-[ai-agents-scores]
-Added new “ai agents” section in ai-agents-scores website, so the admin can see all the ai agents prompt and edit however wants (created 2 workflows in n8n for that task, with two webhooks, POST to update(edit) the ai agents prompts, and GET for reading and showing the prompts in the website)</t>
+          <t>In the AI Agents Score project:
+Added a multi-criteria feedback display, editable ticket levels and per-criterion justification copy buttons.
+Fixed the blank dashboard that sometimes loaded zero tickets.
+Replaced the broken localStorage cache with IndexedDB and added automatic retries.
+Deleted unnecessary code, files, folders, variables, comments and functions, and cleaned up the codebase.</t>
         </is>
       </c>
     </row>
     <row r="185" ht="72" customHeight="1">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>24/08/2026 15:57:23</t>
+          <t>25/08/2026 16:05:00</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
         <is>
-          <t>In ai-agents-scores project:
-Added Multi-criteria feedback display, editable ticket levels, per-criterion justification copy buttons.
-Fixed the blank dashboard that sometimes loaded zero tickets.
-Replaced the broken localStorage cache with IndexedDB and added automatic retries.
-Deleted unnecessary code, files, folders, variables, comments, functions, etc. Cleaned up the codebase.</t>
+          <t>Created a new AI agentic workflow in n8n that retrieves new Gmail messages, parses them and extracts the tracking codes and order numbers (IDs), and collects everything into a dedicated Google Sheet together with the sender's email, the date and time, the sender, the recipient, the order ID, the tracking code, and so on. All of this information is stored, and the workflow is triggered every minute in order to update the Google Sheets list.</t>
         </is>
       </c>
     </row>
     <row r="186" ht="57.6" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>25/08/2026 16:05:00</t>
+          <t>26/08/2026 14:57:29</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
         <is>
-          <t>made new AI agentic workflow in n8n, with gets the new gmail messages, parses and gets the tracking codes(numbers) and order numbers(ids) and collecting that all into the special created google sheets, with the sender email, date-time, email from, email to, order id, tracking code, etc.. all the info has been storing and every 1 minute the workflow is being triggered and updating the google sheets list</t>
+          <t>Updated the AI agentic n8n workflow for the automation of ONEX's Buy For Me service in Gmail, regarding the tracking code and the order ID/number.</t>
         </is>
       </c>
     </row>
     <row r="187" ht="28.8" customHeight="1">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>26/08/2026 14:57:29</t>
+          <t>27/08/2026 15:45:55</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
         <is>
-          <t>updated the ai agentic n8n workflow of the ONEX's Buy for me services automation in the gmail about the tracking code and order id/number</t>
+          <t>Added a node that marks processed Gmail messages as unread.
+Fixed the expressions so that they extract the exact courier and title.
+Corrected the sheet routing and decoded the email subject.</t>
         </is>
       </c>
     </row>
     <row r="188" ht="43.2" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>27/08/2026 15:45:55</t>
+          <t>28/08/2026 15:41:14</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
         <is>
-          <t>Added a node to mark processed Gmails as unread.
-Fixed expressions to extract the exact courier and title.
-Corrected the sheet routing and decoded the email subject.</t>
+          <t>[Buy For Me]
+• Created a Telegram bot notification for every updated or added row.
+[Logistics]
+• Created the correct XML file from the XLSX and CSV files.</t>
         </is>
       </c>
     </row>
     <row r="189" ht="86.40000000000001" customHeight="1">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>28/08/2026 15:41:14</t>
+          <t>31/08/2026 14:18:52</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
         <is>
+          <t>[Logistics]
+• Merged the 141 XML files correctly, sent them to the logistics chief and obtained approval that the files are correct.
+[Buy For Me]
+• Added a clickable link for revealing the tracking code from the email (the tracking code viewer button's link).</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="72" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>01/09/2026 19:41:58</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
           <t>[Buy For Me]
-• Make a telegram bot for every updated or added row.
-[Logistics]
-• Make the correct xml file out of xlsx and csv files</t>
-        </is>
-      </c>
-    </row>
+• Removed the «ԳՆԷՆՑՐ ԻՄ ՓՈԽԱՐԵՆ» նոր պատվերի հարցում request, so that it is no longer taken into account.
+• Applied the structure that Rob mentioned in the Buy4Me Telegram bot.
+[FPL Captain]
+• Fixed the "properties not found" issue.
+[ONEX Academy]
+• Fixed the grammatical issue on the ONEX Academy website.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="129.6" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 19:32:50</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>[Buy For Me]
+• Added Rob's new email and made it tracked, with Telegram bot alerts for it as well.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="28.8" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>03/09/2026 19:50:18</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>[Buy For Me]
+• Deleted the email row from the Telegram bot message.
+• Updated the "BFM Request Link" so that it points to the sorted and filtered ONEX Buy For Me admin page.
+[Buy For Me]
+• Updated the Buy For Me AI agent's prompt, so that the agent now sends only the necessary and correct emails with their tracking codes and order IDs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="43.2" customHeight="1">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>04/09/2026 18:06:19</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>[Buy For Me]
+• Continued working on the automated button clicking system.
+[AI Agents Score]
+• Fixed the "view ticket" text: it is still clickable in the same way, but now shows the ticket ID text instead.
+• Added a "copy" button to each text of the AI agent's criteria clarification, plus a "copy all" button: the user ticks the boxes of the corresponding criteria and clicks copy, and all of the selected ones are copied with a clear, well-structured layout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="28.8" customHeight="1">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>07/09/2026 19:11:36</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>[Buy For Me]
+• changed the links of the telegram bot "BFM request link" to the real searched request links with oder id already searching
+[Buy For Me]
+• add "Tracking code found!" alert in the telegram bot message
+[Buy For Me]
+• return back the sender name in the telegram bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="86.40000000000001" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>

</xml_diff>